<commit_message>
Eredivisie bijgewerkt 01-05-2026 10:58
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  1 May 2026 om 07:07</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  1 May 2026 om 10:58</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  1 May 2026 om 07:07</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  1 May 2026 om 10:58</t>
         </is>
       </c>
     </row>
@@ -17123,9 +17123,9 @@
           <t>1-1</t>
         </is>
       </c>
-      <c r="O19" s="35" t="inlineStr">
-        <is>
-          <t>0-2</t>
+      <c r="O19" s="37" t="inlineStr">
+        <is>
+          <t>·</t>
         </is>
       </c>
       <c r="P19" s="37" t="inlineStr">

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 02-05-2026 10:12
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  1 May 2026 om 10:58</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  2 May 2026 om 10:12</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  1 May 2026 om 10:58</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  2 May 2026 om 10:12</t>
         </is>
       </c>
     </row>
@@ -17123,9 +17123,9 @@
           <t>1-1</t>
         </is>
       </c>
-      <c r="O19" s="37" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="O19" s="35" t="inlineStr">
+        <is>
+          <t>0-2</t>
         </is>
       </c>
       <c r="P19" s="37" t="inlineStr">

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 03-05-2026 10:33
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  2 May 2026 om 10:12</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  3 May 2026 om 10:33</t>
         </is>
       </c>
     </row>
@@ -990,25 +990,25 @@
         </is>
       </c>
       <c r="C3" s="5" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D3" s="5" t="n">
         <v>25</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>4</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
@@ -1017,7 +1017,7 @@
       </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>81%</t>
+          <t>78%</t>
         </is>
       </c>
     </row>
@@ -1072,25 +1072,25 @@
         </is>
       </c>
       <c r="C5" s="10" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D5" s="10" t="n">
         <v>15</v>
       </c>
       <c r="E5" s="10" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F5" s="10" t="n">
         <v>6</v>
       </c>
       <c r="G5" s="11" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J5" s="12" t="inlineStr">
         <is>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>48%</t>
+          <t>47%</t>
         </is>
       </c>
     </row>
@@ -1113,25 +1113,25 @@
         </is>
       </c>
       <c r="C6" s="10" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D6" s="10" t="n">
         <v>14</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F6" s="10" t="n">
         <v>5</v>
       </c>
       <c r="G6" s="11" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
@@ -1140,7 +1140,7 @@
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>45%</t>
+          <t>44%</t>
         </is>
       </c>
     </row>
@@ -1191,38 +1191,38 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>SC Heerenveen</t>
         </is>
       </c>
       <c r="C8" s="10" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D8" s="10" t="n">
         <v>14</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F8" s="10" t="n">
         <v>10</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="J8" s="12" t="inlineStr">
         <is>
-          <t>+7</t>
+          <t>+5</t>
         </is>
       </c>
       <c r="K8" s="10" t="inlineStr">
         <is>
-          <t>45%</t>
+          <t>44%</t>
         </is>
       </c>
     </row>
@@ -1232,38 +1232,38 @@
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>SC Heerenveen</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
         <v>31</v>
       </c>
       <c r="D9" s="15" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E9" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F9" s="15" t="n">
         <v>10</v>
       </c>
       <c r="G9" s="16" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="I9" s="15" t="n">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="J9" s="17" t="inlineStr">
         <is>
-          <t>+4</t>
+          <t>+7</t>
         </is>
       </c>
       <c r="K9" s="15" t="inlineStr">
         <is>
-          <t>42%</t>
+          <t>45%</t>
         </is>
       </c>
     </row>
@@ -1277,10 +1277,10 @@
         </is>
       </c>
       <c r="C10" s="20" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D10" s="20" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E10" s="20" t="n">
         <v>8</v>
@@ -1289,22 +1289,22 @@
         <v>11</v>
       </c>
       <c r="G10" s="21" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H10" s="20" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="I10" s="20" t="n">
         <v>41</v>
       </c>
       <c r="J10" s="22" t="inlineStr">
         <is>
-          <t>+8</t>
+          <t>+10</t>
         </is>
       </c>
       <c r="K10" s="20" t="inlineStr">
         <is>
-          <t>39%</t>
+          <t>41%</t>
         </is>
       </c>
     </row>
@@ -1318,7 +1318,7 @@
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D11" s="15" t="n">
         <v>12</v>
@@ -1327,25 +1327,25 @@
         <v>6</v>
       </c>
       <c r="F11" s="15" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G11" s="16" t="n">
         <v>42</v>
       </c>
       <c r="H11" s="15" t="n">
+        <v>45</v>
+      </c>
+      <c r="I11" s="15" t="n">
         <v>43</v>
       </c>
-      <c r="I11" s="15" t="n">
-        <v>40</v>
-      </c>
       <c r="J11" s="17" t="inlineStr">
         <is>
-          <t>+3</t>
+          <t>+2</t>
         </is>
       </c>
       <c r="K11" s="15" t="inlineStr">
         <is>
-          <t>39%</t>
+          <t>38%</t>
         </is>
       </c>
     </row>
@@ -1478,38 +1478,38 @@
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>PEC Zwolle</t>
+          <t>SBV Excelsior</t>
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D15" s="15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F15" s="15" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="G15" s="16" t="n">
         <v>34</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="I15" s="15" t="n">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="J15" s="24" t="inlineStr">
         <is>
-          <t>-25</t>
+          <t>-14</t>
         </is>
       </c>
       <c r="K15" s="15" t="inlineStr">
         <is>
-          <t>26%</t>
+          <t>28%</t>
         </is>
       </c>
     </row>
@@ -1519,7 +1519,7 @@
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>SBV Excelsior</t>
+          <t>PEC Zwolle</t>
         </is>
       </c>
       <c r="C16" s="20" t="n">
@@ -1529,23 +1529,23 @@
         <v>8</v>
       </c>
       <c r="E16" s="20" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F16" s="20" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G16" s="21" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="H16" s="20" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="I16" s="20" t="n">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="J16" s="23" t="inlineStr">
         <is>
-          <t>-15</t>
+          <t>-25</t>
         </is>
       </c>
       <c r="K16" s="20" t="inlineStr">
@@ -1560,38 +1560,38 @@
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>FC Volendam</t>
+          <t>Telstar 1963</t>
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D17" s="15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F17" s="15" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G17" s="16" t="n">
         <v>31</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="I17" s="15" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="J17" s="24" t="inlineStr">
         <is>
-          <t>-17</t>
+          <t>-10</t>
         </is>
       </c>
       <c r="K17" s="15" t="inlineStr">
         <is>
-          <t>26%</t>
+          <t>22%</t>
         </is>
       </c>
     </row>
@@ -1601,38 +1601,38 @@
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>Telstar 1963</t>
+          <t>FC Volendam</t>
         </is>
       </c>
       <c r="C18" s="20" t="n">
+        <v>32</v>
+      </c>
+      <c r="D18" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="E18" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="F18" s="20" t="n">
+        <v>17</v>
+      </c>
+      <c r="G18" s="21" t="n">
         <v>31</v>
       </c>
-      <c r="D18" s="20" t="n">
-        <v>7</v>
-      </c>
-      <c r="E18" s="20" t="n">
-        <v>9</v>
-      </c>
-      <c r="F18" s="20" t="n">
-        <v>15</v>
-      </c>
-      <c r="G18" s="21" t="n">
-        <v>30</v>
-      </c>
       <c r="H18" s="20" t="n">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="I18" s="20" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="J18" s="23" t="inlineStr">
         <is>
-          <t>-10</t>
+          <t>-18</t>
         </is>
       </c>
       <c r="K18" s="20" t="inlineStr">
         <is>
-          <t>23%</t>
+          <t>25%</t>
         </is>
       </c>
     </row>
@@ -1646,7 +1646,7 @@
         </is>
       </c>
       <c r="C19" s="27" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D19" s="27" t="n">
         <v>5</v>
@@ -1655,7 +1655,7 @@
         <v>10</v>
       </c>
       <c r="F19" s="27" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G19" s="28" t="n">
         <v>25</v>
@@ -1664,11 +1664,11 @@
         <v>30</v>
       </c>
       <c r="I19" s="27" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="J19" s="29" t="inlineStr">
         <is>
-          <t>-23</t>
+          <t>-25</t>
         </is>
       </c>
       <c r="K19" s="27" t="inlineStr">
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  2 May 2026 om 10:12</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  3 May 2026 om 10:33</t>
         </is>
       </c>
     </row>
@@ -15571,9 +15571,9 @@
           <t>3-1</t>
         </is>
       </c>
-      <c r="O3" s="37" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="O3" s="38" t="inlineStr">
+        <is>
+          <t>2-2</t>
         </is>
       </c>
       <c r="P3" s="35" t="inlineStr">
@@ -15770,9 +15770,9 @@
           <t>1-2</t>
         </is>
       </c>
-      <c r="P5" s="37" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="P5" s="35" t="inlineStr">
+        <is>
+          <t>2-3</t>
         </is>
       </c>
       <c r="Q5" s="36" t="inlineStr">
@@ -15944,9 +15944,9 @@
           <t>4-0</t>
         </is>
       </c>
-      <c r="L7" s="37" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="L7" s="36" t="inlineStr">
+        <is>
+          <t>2-0</t>
         </is>
       </c>
       <c r="M7" s="36" t="inlineStr">
@@ -16658,9 +16658,9 @@
           <t>3-1</t>
         </is>
       </c>
-      <c r="S14" s="37" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="S14" s="38" t="inlineStr">
+        <is>
+          <t>1-1</t>
         </is>
       </c>
     </row>
@@ -33729,13 +33729,13 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 04-05-2026 12:15
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -333,10 +333,10 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  3 May 2026 om 10:33</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  4 May 2026 om 12:15</t>
         </is>
       </c>
     </row>
@@ -1031,10 +1031,10 @@
         </is>
       </c>
       <c r="C4" s="10" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D4" s="10" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E4" s="10" t="n">
         <v>7</v>
@@ -1043,22 +1043,22 @@
         <v>7</v>
       </c>
       <c r="G4" s="11" t="n">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="I4" s="10" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J4" s="12" t="inlineStr">
         <is>
-          <t>+23</t>
+          <t>+24</t>
         </is>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>55%</t>
+          <t>56%</t>
         </is>
       </c>
     </row>
@@ -1154,25 +1154,25 @@
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D7" s="10" t="n">
         <v>14</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F7" s="10" t="n">
         <v>5</v>
       </c>
       <c r="G7" s="11" t="n">
+        <v>55</v>
+      </c>
+      <c r="H7" s="10" t="n">
         <v>54</v>
       </c>
-      <c r="H7" s="10" t="n">
-        <v>52</v>
-      </c>
       <c r="I7" s="10" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="J7" s="12" t="inlineStr">
         <is>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="K7" s="10" t="inlineStr">
         <is>
-          <t>45%</t>
+          <t>44%</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>SC Heerenveen</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="C8" s="10" t="n">
@@ -1210,14 +1210,14 @@
         <v>50</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="J8" s="12" t="inlineStr">
         <is>
-          <t>+5</t>
+          <t>+7</t>
         </is>
       </c>
       <c r="K8" s="10" t="inlineStr">
@@ -1232,38 +1232,38 @@
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>SC Heerenveen</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D9" s="15" t="n">
         <v>14</v>
       </c>
       <c r="E9" s="15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F9" s="15" t="n">
         <v>10</v>
       </c>
       <c r="G9" s="16" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="I9" s="15" t="n">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="J9" s="17" t="inlineStr">
         <is>
-          <t>+7</t>
+          <t>+6</t>
         </is>
       </c>
       <c r="K9" s="15" t="inlineStr">
         <is>
-          <t>45%</t>
+          <t>44%</t>
         </is>
       </c>
     </row>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>FC Groningen</t>
+          <t>Sparta Rotterdam</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
@@ -1324,23 +1324,23 @@
         <v>12</v>
       </c>
       <c r="E11" s="15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F11" s="15" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G11" s="16" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="I11" s="15" t="n">
-        <v>43</v>
-      </c>
-      <c r="J11" s="17" t="inlineStr">
-        <is>
-          <t>+2</t>
+        <v>55</v>
+      </c>
+      <c r="J11" s="23" t="inlineStr">
+        <is>
+          <t>-17</t>
         </is>
       </c>
       <c r="K11" s="15" t="inlineStr">
@@ -1355,11 +1355,11 @@
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>Sparta Rotterdam</t>
+          <t>FC Groningen</t>
         </is>
       </c>
       <c r="C12" s="20" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D12" s="20" t="n">
         <v>12</v>
@@ -1368,25 +1368,25 @@
         <v>6</v>
       </c>
       <c r="F12" s="20" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G12" s="21" t="n">
         <v>42</v>
       </c>
       <c r="H12" s="20" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="I12" s="20" t="n">
-        <v>53</v>
-      </c>
-      <c r="J12" s="23" t="inlineStr">
-        <is>
-          <t>-17</t>
+        <v>43</v>
+      </c>
+      <c r="J12" s="22" t="inlineStr">
+        <is>
+          <t>+2</t>
         </is>
       </c>
       <c r="K12" s="20" t="inlineStr">
         <is>
-          <t>39%</t>
+          <t>38%</t>
         </is>
       </c>
     </row>
@@ -1400,25 +1400,25 @@
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D13" s="15" t="n">
         <v>8</v>
       </c>
       <c r="E13" s="15" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F13" s="15" t="n">
         <v>10</v>
       </c>
       <c r="G13" s="16" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="I13" s="15" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J13" s="17" t="inlineStr">
         <is>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="K13" s="15" t="inlineStr">
         <is>
-          <t>26%</t>
+          <t>25%</t>
         </is>
       </c>
     </row>
@@ -1437,38 +1437,38 @@
       </c>
       <c r="B14" s="19" t="inlineStr">
         <is>
-          <t>Fortuna Sittard</t>
+          <t>PEC Zwolle</t>
         </is>
       </c>
       <c r="C14" s="20" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D14" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="E14" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="E14" s="20" t="n">
-        <v>6</v>
-      </c>
       <c r="F14" s="20" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G14" s="21" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H14" s="20" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="I14" s="20" t="n">
-        <v>57</v>
-      </c>
-      <c r="J14" s="23" t="inlineStr">
-        <is>
-          <t>-12</t>
+        <v>66</v>
+      </c>
+      <c r="J14" s="24" t="inlineStr">
+        <is>
+          <t>-24</t>
         </is>
       </c>
       <c r="K14" s="20" t="inlineStr">
         <is>
-          <t>32%</t>
+          <t>28%</t>
         </is>
       </c>
     </row>
@@ -1478,38 +1478,38 @@
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>SBV Excelsior</t>
+          <t>Fortuna Sittard</t>
         </is>
       </c>
       <c r="C15" s="15" t="n">
         <v>32</v>
       </c>
       <c r="D15" s="15" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>16</v>
       </c>
       <c r="G15" s="16" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="I15" s="15" t="n">
-        <v>53</v>
-      </c>
-      <c r="J15" s="24" t="inlineStr">
-        <is>
-          <t>-14</t>
+        <v>59</v>
+      </c>
+      <c r="J15" s="23" t="inlineStr">
+        <is>
+          <t>-13</t>
         </is>
       </c>
       <c r="K15" s="15" t="inlineStr">
         <is>
-          <t>28%</t>
+          <t>31%</t>
         </is>
       </c>
     </row>
@@ -1519,38 +1519,38 @@
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>PEC Zwolle</t>
+          <t>SBV Excelsior</t>
         </is>
       </c>
       <c r="C16" s="20" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D16" s="20" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E16" s="20" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="F16" s="20" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="G16" s="21" t="n">
         <v>34</v>
       </c>
       <c r="H16" s="20" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="I16" s="20" t="n">
-        <v>66</v>
-      </c>
-      <c r="J16" s="23" t="inlineStr">
-        <is>
-          <t>-25</t>
+        <v>53</v>
+      </c>
+      <c r="J16" s="24" t="inlineStr">
+        <is>
+          <t>-14</t>
         </is>
       </c>
       <c r="K16" s="20" t="inlineStr">
         <is>
-          <t>26%</t>
+          <t>28%</t>
         </is>
       </c>
     </row>
@@ -1584,7 +1584,7 @@
       <c r="I17" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-10</t>
         </is>
@@ -1623,11 +1623,11 @@
         <v>33</v>
       </c>
       <c r="I18" s="20" t="n">
-        <v>51</v>
-      </c>
-      <c r="J18" s="23" t="inlineStr">
-        <is>
-          <t>-18</t>
+        <v>52</v>
+      </c>
+      <c r="J18" s="24" t="inlineStr">
+        <is>
+          <t>-19</t>
         </is>
       </c>
       <c r="K18" s="20" t="inlineStr">
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="C20" s="27" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D20" s="27" t="n">
         <v>5</v>
@@ -1696,7 +1696,7 @@
         <v>4</v>
       </c>
       <c r="F20" s="27" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G20" s="28" t="n">
         <v>19</v>
@@ -1705,11 +1705,11 @@
         <v>34</v>
       </c>
       <c r="I20" s="27" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="J20" s="29" t="inlineStr">
         <is>
-          <t>-45</t>
+          <t>-46</t>
         </is>
       </c>
       <c r="K20" s="27" t="inlineStr">
@@ -4066,7 +4066,7 @@
       <c r="I11" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J11" s="24" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-11</t>
         </is>
@@ -4107,7 +4107,7 @@
       <c r="I12" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -4148,7 +4148,7 @@
       <c r="I13" s="15" t="n">
         <v>58</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-8</t>
         </is>
@@ -4189,7 +4189,7 @@
       <c r="I14" s="20" t="n">
         <v>49</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-6</t>
         </is>
@@ -4230,7 +4230,7 @@
       <c r="I15" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -4271,7 +4271,7 @@
       <c r="I16" s="20" t="n">
         <v>68</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-28</t>
         </is>
@@ -4312,7 +4312,7 @@
       <c r="I17" s="15" t="n">
         <v>55</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -4353,7 +4353,7 @@
       <c r="I18" s="20" t="n">
         <v>68</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-28</t>
         </is>
@@ -6794,7 +6794,7 @@
       <c r="I11" s="15" t="n">
         <v>41</v>
       </c>
-      <c r="J11" s="24" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
@@ -6835,7 +6835,7 @@
       <c r="I12" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
@@ -6917,7 +6917,7 @@
       <c r="I14" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -6958,7 +6958,7 @@
       <c r="I15" s="15" t="n">
         <v>55</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -6999,7 +6999,7 @@
       <c r="I16" s="20" t="n">
         <v>52</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-23</t>
         </is>
@@ -7040,7 +7040,7 @@
       <c r="I17" s="15" t="n">
         <v>51</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-27</t>
         </is>
@@ -7081,7 +7081,7 @@
       <c r="I18" s="20" t="n">
         <v>46</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-12</t>
         </is>
@@ -9440,7 +9440,7 @@
       <c r="I9" s="15" t="n">
         <v>68</v>
       </c>
-      <c r="J9" s="24" t="inlineStr">
+      <c r="J9" s="23" t="inlineStr">
         <is>
           <t>-7</t>
         </is>
@@ -9481,7 +9481,7 @@
       <c r="I10" s="20" t="n">
         <v>41</v>
       </c>
-      <c r="J10" s="23" t="inlineStr">
+      <c r="J10" s="24" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -9522,7 +9522,7 @@
       <c r="I11" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="J11" s="24" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-5</t>
         </is>
@@ -9563,7 +9563,7 @@
       <c r="I12" s="20" t="n">
         <v>72</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -9604,7 +9604,7 @@
       <c r="I13" s="15" t="n">
         <v>73</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -9645,7 +9645,7 @@
       <c r="I14" s="20" t="n">
         <v>63</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-16</t>
         </is>
@@ -9686,7 +9686,7 @@
       <c r="I15" s="15" t="n">
         <v>57</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -9727,7 +9727,7 @@
       <c r="I16" s="20" t="n">
         <v>72</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-31</t>
         </is>
@@ -9768,7 +9768,7 @@
       <c r="I17" s="15" t="n">
         <v>80</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-30</t>
         </is>
@@ -9809,7 +9809,7 @@
       <c r="I18" s="20" t="n">
         <v>79</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-33</t>
         </is>
@@ -12168,7 +12168,7 @@
       <c r="I9" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J9" s="24" t="inlineStr">
+      <c r="J9" s="23" t="inlineStr">
         <is>
           <t>-8</t>
         </is>
@@ -12209,7 +12209,7 @@
       <c r="I10" s="20" t="n">
         <v>53</v>
       </c>
-      <c r="J10" s="23" t="inlineStr">
+      <c r="J10" s="24" t="inlineStr">
         <is>
           <t>-5</t>
         </is>
@@ -12250,7 +12250,7 @@
       <c r="I11" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J11" s="24" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-12</t>
         </is>
@@ -12291,7 +12291,7 @@
       <c r="I12" s="20" t="n">
         <v>64</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -12332,7 +12332,7 @@
       <c r="I13" s="15" t="n">
         <v>56</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -12414,7 +12414,7 @@
       <c r="I15" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -12455,7 +12455,7 @@
       <c r="I16" s="20" t="n">
         <v>57</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-16</t>
         </is>
@@ -12496,7 +12496,7 @@
       <c r="I17" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -12537,7 +12537,7 @@
       <c r="I18" s="20" t="n">
         <v>69</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-27</t>
         </is>
@@ -14896,7 +14896,7 @@
       <c r="I9" s="15" t="n">
         <v>50</v>
       </c>
-      <c r="J9" s="24" t="inlineStr">
+      <c r="J9" s="23" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -15019,7 +15019,7 @@
       <c r="I12" s="20" t="n">
         <v>55</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -15060,7 +15060,7 @@
       <c r="I13" s="15" t="n">
         <v>59</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -15101,7 +15101,7 @@
       <c r="I14" s="20" t="n">
         <v>60</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -15142,7 +15142,7 @@
       <c r="I15" s="15" t="n">
         <v>44</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -15183,7 +15183,7 @@
       <c r="I16" s="20" t="n">
         <v>67</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-28</t>
         </is>
@@ -15224,7 +15224,7 @@
       <c r="I17" s="15" t="n">
         <v>61</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -15265,7 +15265,7 @@
       <c r="I18" s="20" t="n">
         <v>59</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-27</t>
         </is>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  3 May 2026 om 10:33</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  4 May 2026 om 12:15</t>
         </is>
       </c>
     </row>
@@ -15618,9 +15618,9 @@
           <t>4-1</t>
         </is>
       </c>
-      <c r="E4" s="37" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="E4" s="38" t="inlineStr">
+        <is>
+          <t>2-2</t>
         </is>
       </c>
       <c r="F4" s="36" t="inlineStr">
@@ -16066,9 +16066,9 @@
           <t>1-2</t>
         </is>
       </c>
-      <c r="Q8" s="37" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="Q8" s="35" t="inlineStr">
+        <is>
+          <t>0-2</t>
         </is>
       </c>
       <c r="R8" s="35" t="inlineStr">
@@ -16215,9 +16215,9 @@
           <t>1-0</t>
         </is>
       </c>
-      <c r="H10" s="37" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="H10" s="35" t="inlineStr">
+        <is>
+          <t>1-2</t>
         </is>
       </c>
       <c r="I10" s="34" t="inlineStr">
@@ -16715,9 +16715,9 @@
           <t>0-2</t>
         </is>
       </c>
-      <c r="K15" s="37" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="K15" s="36" t="inlineStr">
+        <is>
+          <t>1-0</t>
         </is>
       </c>
       <c r="L15" s="36" t="inlineStr">
@@ -17098,9 +17098,9 @@
           <t>1-1</t>
         </is>
       </c>
-      <c r="J19" s="37" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="J19" s="38" t="inlineStr">
+        <is>
+          <t>2-2</t>
         </is>
       </c>
       <c r="K19" s="36" t="inlineStr">
@@ -19520,7 +19520,7 @@
       <c r="I9" s="15" t="n">
         <v>48</v>
       </c>
-      <c r="J9" s="24" t="inlineStr">
+      <c r="J9" s="23" t="inlineStr">
         <is>
           <t>-7</t>
         </is>
@@ -19643,7 +19643,7 @@
       <c r="I12" s="20" t="n">
         <v>42</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>-5</t>
         </is>
@@ -19684,7 +19684,7 @@
       <c r="I13" s="15" t="n">
         <v>49</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-1</t>
         </is>
@@ -19725,7 +19725,7 @@
       <c r="I14" s="20" t="n">
         <v>61</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -19766,7 +19766,7 @@
       <c r="I15" s="15" t="n">
         <v>64</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -19807,7 +19807,7 @@
       <c r="I16" s="20" t="n">
         <v>55</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-21</t>
         </is>
@@ -19848,7 +19848,7 @@
       <c r="I17" s="15" t="n">
         <v>60</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-26</t>
         </is>
@@ -19889,7 +19889,7 @@
       <c r="I18" s="20" t="n">
         <v>53</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -22289,7 +22289,7 @@
       <c r="I10" s="20" t="n">
         <v>53</v>
       </c>
-      <c r="J10" s="23" t="inlineStr">
+      <c r="J10" s="24" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
@@ -22330,7 +22330,7 @@
       <c r="I11" s="15" t="n">
         <v>50</v>
       </c>
-      <c r="J11" s="24" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
@@ -22412,7 +22412,7 @@
       <c r="I13" s="15" t="n">
         <v>62</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -22453,7 +22453,7 @@
       <c r="I14" s="20" t="n">
         <v>56</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-10</t>
         </is>
@@ -22494,7 +22494,7 @@
       <c r="I15" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -22535,7 +22535,7 @@
       <c r="I16" s="20" t="n">
         <v>64</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -22576,7 +22576,7 @@
       <c r="I17" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-16</t>
         </is>
@@ -22617,7 +22617,7 @@
       <c r="I18" s="20" t="n">
         <v>68</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-32</t>
         </is>
@@ -25058,7 +25058,7 @@
       <c r="I11" s="15" t="n">
         <v>64</v>
       </c>
-      <c r="J11" s="24" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -25099,7 +25099,7 @@
       <c r="I12" s="20" t="n">
         <v>65</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -25140,7 +25140,7 @@
       <c r="I13" s="15" t="n">
         <v>49</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -25181,7 +25181,7 @@
       <c r="I14" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-10</t>
         </is>
@@ -25222,7 +25222,7 @@
       <c r="I15" s="15" t="n">
         <v>69</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-24</t>
         </is>
@@ -25263,7 +25263,7 @@
       <c r="I16" s="20" t="n">
         <v>59</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -25304,7 +25304,7 @@
       <c r="I17" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-11</t>
         </is>
@@ -25345,7 +25345,7 @@
       <c r="I18" s="20" t="n">
         <v>64</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-20</t>
         </is>
@@ -27704,7 +27704,7 @@
       <c r="I9" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J9" s="24" t="inlineStr">
+      <c r="J9" s="23" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -27745,7 +27745,7 @@
       <c r="I10" s="20" t="n">
         <v>63</v>
       </c>
-      <c r="J10" s="23" t="inlineStr">
+      <c r="J10" s="24" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -27786,7 +27786,7 @@
       <c r="I11" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="J11" s="24" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -27868,7 +27868,7 @@
       <c r="I13" s="15" t="n">
         <v>55</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -27909,7 +27909,7 @@
       <c r="I14" s="20" t="n">
         <v>71</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -27950,7 +27950,7 @@
       <c r="I15" s="15" t="n">
         <v>56</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-16</t>
         </is>
@@ -27991,7 +27991,7 @@
       <c r="I16" s="20" t="n">
         <v>48</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -28032,7 +28032,7 @@
       <c r="I17" s="15" t="n">
         <v>66</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -28073,7 +28073,7 @@
       <c r="I18" s="20" t="n">
         <v>69</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -30473,7 +30473,7 @@
       <c r="I10" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="J10" s="23" t="inlineStr">
+      <c r="J10" s="24" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
@@ -30514,7 +30514,7 @@
       <c r="I11" s="15" t="n">
         <v>49</v>
       </c>
-      <c r="J11" s="24" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -30555,7 +30555,7 @@
       <c r="I12" s="20" t="n">
         <v>70</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -30596,7 +30596,7 @@
       <c r="I13" s="15" t="n">
         <v>58</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
@@ -30637,7 +30637,7 @@
       <c r="I14" s="20" t="n">
         <v>62</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-10</t>
         </is>
@@ -30678,7 +30678,7 @@
       <c r="I15" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -30719,7 +30719,7 @@
       <c r="I16" s="20" t="n">
         <v>61</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-20</t>
         </is>
@@ -30760,7 +30760,7 @@
       <c r="I17" s="15" t="n">
         <v>67</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-29</t>
         </is>
@@ -30801,7 +30801,7 @@
       <c r="I18" s="20" t="n">
         <v>78</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-36</t>
         </is>
@@ -31346,7 +31346,7 @@
       <c r="I11" s="15" t="n">
         <v>57</v>
       </c>
-      <c r="J11" s="24" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -31387,7 +31387,7 @@
       <c r="I12" s="20" t="n">
         <v>51</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>-8</t>
         </is>
@@ -31428,7 +31428,7 @@
       <c r="I13" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -31469,7 +31469,7 @@
       <c r="I14" s="20" t="n">
         <v>43</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
@@ -31510,7 +31510,7 @@
       <c r="I15" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -31551,7 +31551,7 @@
       <c r="I16" s="20" t="n">
         <v>63</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-21</t>
         </is>
@@ -31592,7 +31592,7 @@
       <c r="I17" s="15" t="n">
         <v>58</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-24</t>
         </is>
@@ -31633,7 +31633,7 @@
       <c r="I18" s="20" t="n">
         <v>56</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -36790,7 +36790,7 @@
       <c r="I12" s="20" t="n">
         <v>56</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -36831,7 +36831,7 @@
       <c r="I13" s="15" t="n">
         <v>70</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -36872,7 +36872,7 @@
       <c r="I14" s="20" t="n">
         <v>67</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -36913,7 +36913,7 @@
       <c r="I15" s="15" t="n">
         <v>59</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-25</t>
         </is>
@@ -36954,7 +36954,7 @@
       <c r="I16" s="20" t="n">
         <v>75</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-34</t>
         </is>
@@ -36995,7 +36995,7 @@
       <c r="I17" s="15" t="n">
         <v>56</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -37036,7 +37036,7 @@
       <c r="I18" s="20" t="n">
         <v>73</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-23</t>
         </is>
@@ -39436,7 +39436,7 @@
       <c r="I10" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J10" s="23" t="inlineStr">
+      <c r="J10" s="24" t="inlineStr">
         <is>
           <t>-6</t>
         </is>
@@ -39477,7 +39477,7 @@
       <c r="I11" s="15" t="n">
         <v>64</v>
       </c>
-      <c r="J11" s="24" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -39518,7 +39518,7 @@
       <c r="I12" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>-5</t>
         </is>
@@ -39559,7 +39559,7 @@
       <c r="I13" s="15" t="n">
         <v>56</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-10</t>
         </is>
@@ -39600,7 +39600,7 @@
       <c r="I14" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
@@ -39641,7 +39641,7 @@
       <c r="I15" s="15" t="n">
         <v>62</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-23</t>
         </is>
@@ -39682,7 +39682,7 @@
       <c r="I16" s="20" t="n">
         <v>71</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-29</t>
         </is>
@@ -39723,7 +39723,7 @@
       <c r="I17" s="15" t="n">
         <v>71</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-39</t>
         </is>
@@ -39764,7 +39764,7 @@
       <c r="I18" s="20" t="n">
         <v>65</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-32</t>
         </is>
@@ -42164,7 +42164,7 @@
       <c r="I10" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J10" s="23" t="inlineStr">
+      <c r="J10" s="24" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -42205,7 +42205,7 @@
       <c r="I11" s="15" t="n">
         <v>70</v>
       </c>
-      <c r="J11" s="24" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -42246,7 +42246,7 @@
       <c r="I12" s="20" t="n">
         <v>51</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>-11</t>
         </is>
@@ -42287,7 +42287,7 @@
       <c r="I13" s="15" t="n">
         <v>52</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -42328,7 +42328,7 @@
       <c r="I14" s="20" t="n">
         <v>55</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -42369,7 +42369,7 @@
       <c r="I15" s="15" t="n">
         <v>51</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -42410,7 +42410,7 @@
       <c r="I16" s="20" t="n">
         <v>48</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -42451,7 +42451,7 @@
       <c r="I17" s="15" t="n">
         <v>67</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-31</t>
         </is>
@@ -42492,7 +42492,7 @@
       <c r="I18" s="20" t="n">
         <v>49</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-16</t>
         </is>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 05-05-2026 11:49
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  4 May 2026 om 12:15</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  5 May 2026 om 11:49</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  4 May 2026 om 12:15</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  5 May 2026 om 11:49</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 06-05-2026 13:19
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  5 May 2026 om 11:49</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  6 May 2026 om 13:19</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  5 May 2026 om 11:49</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  6 May 2026 om 13:19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 07-05-2026 13:19
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  6 May 2026 om 13:19</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  7 May 2026 om 13:19</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  6 May 2026 om 13:19</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  7 May 2026 om 13:19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 08-05-2026 11:56
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  7 May 2026 om 13:19</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  8 May 2026 om 11:56</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  7 May 2026 om 13:19</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  8 May 2026 om 11:56</t>
         </is>
       </c>
     </row>
@@ -16717,7 +16717,7 @@
       </c>
       <c r="K15" s="36" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="L15" s="36" t="inlineStr">
@@ -17123,9 +17123,9 @@
           <t>1-1</t>
         </is>
       </c>
-      <c r="O19" s="35" t="inlineStr">
-        <is>
-          <t>0-2</t>
+      <c r="O19" s="37" t="inlineStr">
+        <is>
+          <t>·</t>
         </is>
       </c>
       <c r="P19" s="37" t="inlineStr">

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 09-05-2026 10:33
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  8 May 2026 om 11:56</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  9 May 2026 om 10:33</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  8 May 2026 om 11:56</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  9 May 2026 om 10:33</t>
         </is>
       </c>
     </row>
@@ -16717,7 +16717,7 @@
       </c>
       <c r="K15" s="36" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="L15" s="36" t="inlineStr">
@@ -17123,9 +17123,9 @@
           <t>1-1</t>
         </is>
       </c>
-      <c r="O19" s="37" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="O19" s="35" t="inlineStr">
+        <is>
+          <t>0-2</t>
         </is>
       </c>
       <c r="P19" s="37" t="inlineStr">

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 10-05-2026 10:48
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  9 May 2026 om 10:33</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  10 May 2026 om 10:48</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  9 May 2026 om 10:33</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  10 May 2026 om 10:48</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 12-05-2026 13:27
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  11 May 2026 om 16:48</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  12 May 2026 om 13:26</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  11 May 2026 om 16:48</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  12 May 2026 om 13:26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 13-05-2026 16:11
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  12 May 2026 om 13:26</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  13 May 2026 om 16:11</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  12 May 2026 om 13:26</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  13 May 2026 om 16:11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 14-05-2026 12:22
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  13 May 2026 om 16:11</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  14 May 2026 om 12:22</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  13 May 2026 om 16:11</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  14 May 2026 om 12:22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 15-05-2026 13:15
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  14 May 2026 om 12:22</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  15 May 2026 om 13:15</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  14 May 2026 om 12:22</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  15 May 2026 om 13:15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 16-05-2026 10:48
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  15 May 2026 om 13:15</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  16 May 2026 om 10:48</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  15 May 2026 om 13:15</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  16 May 2026 om 10:48</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 17-05-2026 10:56
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  16 May 2026 om 10:48</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  17 May 2026 om 10:56</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  16 May 2026 om 10:48</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  17 May 2026 om 10:56</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 18-05-2026 17:18
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  17 May 2026 om 10:56</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  18 May 2026 om 17:18</t>
         </is>
       </c>
     </row>
@@ -990,10 +990,10 @@
         </is>
       </c>
       <c r="C3" s="5" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>3</v>
@@ -1002,17 +1002,17 @@
         <v>4</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>+52</t>
+          <t>+56</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
@@ -1031,10 +1031,10 @@
         </is>
       </c>
       <c r="C4" s="10" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D4" s="10" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E4" s="10" t="n">
         <v>8</v>
@@ -1043,22 +1043,22 @@
         <v>7</v>
       </c>
       <c r="G4" s="11" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I4" s="10" t="n">
         <v>44</v>
       </c>
       <c r="J4" s="12" t="inlineStr">
         <is>
-          <t>+24</t>
+          <t>+26</t>
         </is>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>55%</t>
+          <t>56%</t>
         </is>
       </c>
     </row>
@@ -1068,38 +1068,38 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>FC Twente '65</t>
+          <t>NEC</t>
         </is>
       </c>
       <c r="C5" s="10" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D5" s="10" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E5" s="10" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F5" s="10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G5" s="11" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>58</v>
+        <v>77</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>35</v>
+        <v>53</v>
       </c>
       <c r="J5" s="12" t="inlineStr">
         <is>
-          <t>+23</t>
+          <t>+24</t>
         </is>
       </c>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>45%</t>
+          <t>47%</t>
         </is>
       </c>
     </row>
@@ -1109,38 +1109,38 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>NEC</t>
+          <t>FC Twente '65</t>
         </is>
       </c>
       <c r="C6" s="10" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D6" s="10" t="n">
         <v>15</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F6" s="10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G6" s="11" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>75</v>
+        <v>59</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>52</v>
+        <v>40</v>
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
-          <t>+23</t>
+          <t>+19</t>
         </is>
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>45%</t>
+          <t>44%</t>
         </is>
       </c>
     </row>
@@ -1154,19 +1154,19 @@
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D7" s="10" t="n">
         <v>14</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F7" s="10" t="n">
         <v>6</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H7" s="10" t="n">
         <v>62</v>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="K7" s="10" t="inlineStr">
         <is>
-          <t>42%</t>
+          <t>41%</t>
         </is>
       </c>
     </row>
@@ -1191,38 +1191,38 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>FC Utrecht</t>
         </is>
       </c>
       <c r="C8" s="10" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D8" s="10" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F8" s="10" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H8" s="10" t="n">
         <v>55</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="J8" s="12" t="inlineStr">
         <is>
-          <t>+7</t>
+          <t>+13</t>
         </is>
       </c>
       <c r="K8" s="10" t="inlineStr">
         <is>
-          <t>42%</t>
+          <t>44%</t>
         </is>
       </c>
     </row>
@@ -1232,38 +1232,38 @@
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>FC Utrecht</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D9" s="15" t="n">
         <v>14</v>
       </c>
       <c r="E9" s="15" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F9" s="15" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G9" s="16" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="I9" s="15" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="J9" s="17" t="inlineStr">
         <is>
-          <t>+11</t>
+          <t>+7</t>
         </is>
       </c>
       <c r="K9" s="15" t="inlineStr">
         <is>
-          <t>42%</t>
+          <t>41%</t>
         </is>
       </c>
     </row>
@@ -1277,19 +1277,19 @@
         </is>
       </c>
       <c r="C10" s="20" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D10" s="20" t="n">
         <v>14</v>
       </c>
       <c r="E10" s="20" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F10" s="20" t="n">
         <v>11</v>
       </c>
       <c r="G10" s="21" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H10" s="20" t="n">
         <v>57</v>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="K10" s="20" t="inlineStr">
         <is>
-          <t>42%</t>
+          <t>41%</t>
         </is>
       </c>
     </row>
@@ -1318,10 +1318,10 @@
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D11" s="15" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E11" s="15" t="n">
         <v>6</v>
@@ -1330,22 +1330,22 @@
         <v>14</v>
       </c>
       <c r="G11" s="16" t="n">
+        <v>48</v>
+      </c>
+      <c r="H11" s="15" t="n">
+        <v>49</v>
+      </c>
+      <c r="I11" s="15" t="n">
         <v>45</v>
       </c>
-      <c r="H11" s="15" t="n">
-        <v>47</v>
-      </c>
-      <c r="I11" s="15" t="n">
-        <v>44</v>
-      </c>
       <c r="J11" s="17" t="inlineStr">
         <is>
-          <t>+3</t>
+          <t>+4</t>
         </is>
       </c>
       <c r="K11" s="15" t="inlineStr">
         <is>
-          <t>39%</t>
+          <t>41%</t>
         </is>
       </c>
     </row>
@@ -1359,7 +1359,7 @@
         </is>
       </c>
       <c r="C12" s="20" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D12" s="20" t="n">
         <v>12</v>
@@ -1368,25 +1368,25 @@
         <v>7</v>
       </c>
       <c r="F12" s="20" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G12" s="21" t="n">
         <v>43</v>
       </c>
       <c r="H12" s="20" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="I12" s="20" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="J12" s="23" t="inlineStr">
         <is>
-          <t>-21</t>
+          <t>-22</t>
         </is>
       </c>
       <c r="K12" s="20" t="inlineStr">
         <is>
-          <t>36%</t>
+          <t>35%</t>
         </is>
       </c>
     </row>
@@ -1400,7 +1400,7 @@
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D13" s="15" t="n">
         <v>11</v>
@@ -1409,7 +1409,7 @@
         <v>6</v>
       </c>
       <c r="F13" s="15" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G13" s="16" t="n">
         <v>39</v>
@@ -1418,16 +1418,16 @@
         <v>49</v>
       </c>
       <c r="I13" s="15" t="n">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="J13" s="24" t="inlineStr">
         <is>
-          <t>-12</t>
+          <t>-14</t>
         </is>
       </c>
       <c r="K13" s="15" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>32%</t>
         </is>
       </c>
     </row>
@@ -1441,7 +1441,7 @@
         </is>
       </c>
       <c r="C14" s="20" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D14" s="20" t="n">
         <v>8</v>
@@ -1450,20 +1450,20 @@
         <v>14</v>
       </c>
       <c r="F14" s="20" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G14" s="21" t="n">
         <v>38</v>
       </c>
       <c r="H14" s="20" t="n">
+        <v>54</v>
+      </c>
+      <c r="I14" s="20" t="n">
         <v>53</v>
       </c>
-      <c r="I14" s="20" t="n">
-        <v>51</v>
-      </c>
       <c r="J14" s="22" t="inlineStr">
         <is>
-          <t>+2</t>
+          <t>+1</t>
         </is>
       </c>
       <c r="K14" s="20" t="inlineStr">
@@ -1478,38 +1478,38 @@
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>PEC Zwolle</t>
+          <t>SBV Excelsior</t>
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D15" s="15" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F15" s="15" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G15" s="16" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I15" s="15" t="n">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="J15" s="24" t="inlineStr">
         <is>
-          <t>-25</t>
+          <t>-13</t>
         </is>
       </c>
       <c r="K15" s="15" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>29%</t>
         </is>
       </c>
     </row>
@@ -1519,38 +1519,38 @@
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>SBV Excelsior</t>
+          <t>Telstar 1963</t>
         </is>
       </c>
       <c r="C16" s="20" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D16" s="20" t="n">
         <v>9</v>
       </c>
       <c r="E16" s="20" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F16" s="20" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G16" s="21" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H16" s="20" t="n">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="I16" s="20" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="J16" s="23" t="inlineStr">
         <is>
-          <t>-14</t>
+          <t>-6</t>
         </is>
       </c>
       <c r="K16" s="20" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>26%</t>
         </is>
       </c>
     </row>
@@ -1560,14 +1560,14 @@
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>Telstar 1963</t>
+          <t>PEC Zwolle</t>
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D17" s="15" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E17" s="15" t="n">
         <v>10</v>
@@ -1576,22 +1576,22 @@
         <v>15</v>
       </c>
       <c r="G17" s="16" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="I17" s="15" t="n">
-        <v>54</v>
+        <v>71</v>
       </c>
       <c r="J17" s="24" t="inlineStr">
         <is>
-          <t>-7</t>
+          <t>-27</t>
         </is>
       </c>
       <c r="K17" s="15" t="inlineStr">
         <is>
-          <t>24%</t>
+          <t>26%</t>
         </is>
       </c>
     </row>
@@ -1605,7 +1605,7 @@
         </is>
       </c>
       <c r="C18" s="20" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D18" s="20" t="n">
         <v>8</v>
@@ -1614,20 +1614,20 @@
         <v>8</v>
       </c>
       <c r="F18" s="20" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G18" s="21" t="n">
         <v>32</v>
       </c>
       <c r="H18" s="20" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I18" s="20" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="J18" s="23" t="inlineStr">
         <is>
-          <t>-19</t>
+          <t>-20</t>
         </is>
       </c>
       <c r="K18" s="20" t="inlineStr">
@@ -1646,25 +1646,25 @@
         </is>
       </c>
       <c r="C19" s="27" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D19" s="27" t="n">
         <v>6</v>
       </c>
       <c r="E19" s="27" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F19" s="27" t="n">
         <v>17</v>
       </c>
       <c r="G19" s="28" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H19" s="27" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="I19" s="27" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="J19" s="29" t="inlineStr">
         <is>
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="C20" s="27" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D20" s="27" t="n">
         <v>5</v>
@@ -1696,20 +1696,20 @@
         <v>4</v>
       </c>
       <c r="F20" s="27" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G20" s="28" t="n">
         <v>19</v>
       </c>
       <c r="H20" s="27" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I20" s="27" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="J20" s="29" t="inlineStr">
         <is>
-          <t>-49</t>
+          <t>-50</t>
         </is>
       </c>
       <c r="K20" s="27" t="inlineStr">
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  17 May 2026 om 10:56</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  18 May 2026 om 17:18</t>
         </is>
       </c>
     </row>
@@ -15653,9 +15653,9 @@
           <t>4-0</t>
         </is>
       </c>
-      <c r="L4" s="39" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="L4" s="37" t="inlineStr">
+        <is>
+          <t>3-3</t>
         </is>
       </c>
       <c r="M4" s="35" t="inlineStr">
@@ -15929,9 +15929,9 @@
           <t>0-1</t>
         </is>
       </c>
-      <c r="I7" s="39" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="I7" s="36" t="inlineStr">
+        <is>
+          <t>2-0</t>
         </is>
       </c>
       <c r="J7" s="36" t="inlineStr">
@@ -16076,9 +16076,9 @@
           <t>0-1</t>
         </is>
       </c>
-      <c r="S8" s="39" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="S8" s="35" t="inlineStr">
+        <is>
+          <t>1-2</t>
         </is>
       </c>
     </row>
@@ -16389,9 +16389,9 @@
           <t>1-2</t>
         </is>
       </c>
-      <c r="D12" s="39" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="D12" s="35" t="inlineStr">
+        <is>
+          <t>1-2</t>
         </is>
       </c>
       <c r="E12" s="35" t="inlineStr">
@@ -16613,9 +16613,9 @@
           <t>2-3</t>
         </is>
       </c>
-      <c r="J14" s="39" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="J14" s="36" t="inlineStr">
+        <is>
+          <t>2-1</t>
         </is>
       </c>
       <c r="K14" s="36" t="inlineStr">
@@ -16700,9 +16700,9 @@
           <t>1-2</t>
         </is>
       </c>
-      <c r="H15" s="39" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="H15" s="35" t="inlineStr">
+        <is>
+          <t>0-2</t>
         </is>
       </c>
       <c r="I15" s="36" t="inlineStr">
@@ -16782,9 +16782,9 @@
           <t>4-2</t>
         </is>
       </c>
-      <c r="E16" s="39" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="E16" s="36" t="inlineStr">
+        <is>
+          <t>5-1</t>
         </is>
       </c>
       <c r="F16" s="36" t="inlineStr">
@@ -16961,9 +16961,9 @@
           <t>SC Heerenveen</t>
         </is>
       </c>
-      <c r="B18" s="39" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="B18" s="37" t="inlineStr">
+        <is>
+          <t>0-0</t>
         </is>
       </c>
       <c r="C18" s="36" t="inlineStr">
@@ -17128,9 +17128,9 @@
           <t>0-2</t>
         </is>
       </c>
-      <c r="P19" s="39" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="P19" s="35" t="inlineStr">
+        <is>
+          <t>2-3</t>
         </is>
       </c>
       <c r="Q19" s="35" t="inlineStr">
@@ -33729,17 +33729,17 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>+52</t>
+          <t>+56</t>
         </is>
       </c>
       <c r="H5" s="45" t="inlineStr">

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 19-05-2026 17:30
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  18 May 2026 om 17:18</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  19 May 2026 om 17:30</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  18 May 2026 om 17:18</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  19 May 2026 om 17:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 20-05-2026 18:01
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  19 May 2026 om 17:30</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  20 May 2026 om 18:01</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  19 May 2026 om 17:30</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  20 May 2026 om 18:01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 21-05-2026 17:19
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  20 May 2026 om 18:01</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  21 May 2026 om 17:19</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  20 May 2026 om 18:01</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  21 May 2026 om 17:19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 22-05-2026 16:10
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  21 May 2026 om 17:19</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  22 May 2026 om 16:10</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  21 May 2026 om 17:19</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  22 May 2026 om 16:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 23-05-2026 11:38
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  22 May 2026 om 16:10</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  23 May 2026 om 11:38</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  22 May 2026 om 16:10</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  23 May 2026 om 11:38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 24-05-2026 11:50
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  23 May 2026 om 11:38</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  24 May 2026 om 11:50</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  23 May 2026 om 11:38</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  24 May 2026 om 11:50</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 25-05-2026 16:10
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  24 May 2026 om 11:50</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  25 May 2026 om 16:10</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  24 May 2026 om 11:50</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  25 May 2026 om 16:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 26-05-2026 18:06
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  25 May 2026 om 16:10</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  26 May 2026 om 18:06</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  25 May 2026 om 16:10</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  26 May 2026 om 18:06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 27-05-2026 18:07
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -143,13 +143,13 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="FFCCCCCC"/>
+      <i val="1"/>
+      <color rgb="FF888888"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="FF888888"/>
+      <color rgb="FFCCCCCC"/>
       <sz val="9"/>
     </font>
     <font>
@@ -381,11 +381,11 @@
     <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  26 May 2026 om 18:06</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  27 May 2026 om 18:07</t>
         </is>
       </c>
     </row>
@@ -3607,7 +3607,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="40" t="inlineStr">
+      <c r="A22" s="39" t="inlineStr">
         <is>
           <t>🟢 Groen = Thuiswinst   🔴 Rood = Thuisverlies   🟡 Geel = Gelijk   · = Niet gespeeld</t>
         </is>
@@ -6335,7 +6335,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="40" t="inlineStr">
+      <c r="A22" s="39" t="inlineStr">
         <is>
           <t>🟢 Groen = Thuiswinst   🔴 Rood = Thuisverlies   🟡 Geel = Gelijk   · = Niet gespeeld</t>
         </is>
@@ -7337,7 +7337,7 @@
           <t>0-2</t>
         </is>
       </c>
-      <c r="E3" s="39" t="inlineStr">
+      <c r="E3" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -7357,12 +7357,12 @@
           <t>2-4</t>
         </is>
       </c>
-      <c r="I3" s="39" t="inlineStr">
+      <c r="I3" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="J3" s="39" t="inlineStr">
+      <c r="J3" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -7372,7 +7372,7 @@
           <t>0-0</t>
         </is>
       </c>
-      <c r="L3" s="39" t="inlineStr">
+      <c r="L3" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -7449,12 +7449,12 @@
           <t>3-0</t>
         </is>
       </c>
-      <c r="H4" s="39" t="inlineStr">
+      <c r="H4" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="I4" s="39" t="inlineStr">
+      <c r="I4" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -7474,7 +7474,7 @@
           <t>2-0</t>
         </is>
       </c>
-      <c r="M4" s="39" t="inlineStr">
+      <c r="M4" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -7494,7 +7494,7 @@
           <t>1-0</t>
         </is>
       </c>
-      <c r="Q4" s="39" t="inlineStr">
+      <c r="Q4" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -7541,7 +7541,7 @@
           <t>2-0</t>
         </is>
       </c>
-      <c r="G5" s="39" t="inlineStr">
+      <c r="G5" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -7566,7 +7566,7 @@
           <t>4-1</t>
         </is>
       </c>
-      <c r="L5" s="39" t="inlineStr">
+      <c r="L5" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -7586,12 +7586,12 @@
           <t>2-1</t>
         </is>
       </c>
-      <c r="P5" s="39" t="inlineStr">
+      <c r="P5" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="Q5" s="39" t="inlineStr">
+      <c r="Q5" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -7618,12 +7618,12 @@
           <t>3-0</t>
         </is>
       </c>
-      <c r="C6" s="39" t="inlineStr">
+      <c r="C6" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="D6" s="39" t="inlineStr">
+      <c r="D6" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -7643,7 +7643,7 @@
           <t>2-0</t>
         </is>
       </c>
-      <c r="H6" s="39" t="inlineStr">
+      <c r="H6" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -7673,7 +7673,7 @@
           <t>1-1</t>
         </is>
       </c>
-      <c r="N6" s="39" t="inlineStr">
+      <c r="N6" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -7710,12 +7710,12 @@
           <t>FC Groningen</t>
         </is>
       </c>
-      <c r="B7" s="39" t="inlineStr">
+      <c r="B7" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="C7" s="39" t="inlineStr">
+      <c r="C7" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -7750,7 +7750,7 @@
           <t>1-1</t>
         </is>
       </c>
-      <c r="J7" s="39" t="inlineStr">
+      <c r="J7" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -7795,7 +7795,7 @@
           <t>2-0</t>
         </is>
       </c>
-      <c r="S7" s="39" t="inlineStr">
+      <c r="S7" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -7807,7 +7807,7 @@
           <t>FC Twente</t>
         </is>
       </c>
-      <c r="B8" s="39" t="inlineStr">
+      <c r="B8" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -7842,12 +7842,12 @@
           <t>3-1</t>
         </is>
       </c>
-      <c r="I8" s="39" t="inlineStr">
+      <c r="I8" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="J8" s="39" t="inlineStr">
+      <c r="J8" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -7877,7 +7877,7 @@
           <t>2-0</t>
         </is>
       </c>
-      <c r="P8" s="39" t="inlineStr">
+      <c r="P8" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -7914,7 +7914,7 @@
           <t>0-0</t>
         </is>
       </c>
-      <c r="D9" s="39" t="inlineStr">
+      <c r="D9" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -7924,7 +7924,7 @@
           <t>3-3</t>
         </is>
       </c>
-      <c r="F9" s="39" t="inlineStr">
+      <c r="F9" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -7949,7 +7949,7 @@
           <t>6-0</t>
         </is>
       </c>
-      <c r="K9" s="39" t="inlineStr">
+      <c r="K9" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -7979,7 +7979,7 @@
           <t>1-2</t>
         </is>
       </c>
-      <c r="Q9" s="39" t="inlineStr">
+      <c r="Q9" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -7989,7 +7989,7 @@
           <t>2-0</t>
         </is>
       </c>
-      <c r="S9" s="39" t="inlineStr">
+      <c r="S9" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8011,7 +8011,7 @@
           <t>0-3</t>
         </is>
       </c>
-      <c r="D10" s="39" t="inlineStr">
+      <c r="D10" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8021,7 +8021,7 @@
           <t>3-3</t>
         </is>
       </c>
-      <c r="F10" s="39" t="inlineStr">
+      <c r="F10" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8071,12 +8071,12 @@
           <t>2-2</t>
         </is>
       </c>
-      <c r="P10" s="39" t="inlineStr">
+      <c r="P10" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="Q10" s="39" t="inlineStr">
+      <c r="Q10" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8103,12 +8103,12 @@
           <t>1-0</t>
         </is>
       </c>
-      <c r="C11" s="39" t="inlineStr">
+      <c r="C11" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="D11" s="39" t="inlineStr">
+      <c r="D11" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8128,7 +8128,7 @@
           <t>2-3</t>
         </is>
       </c>
-      <c r="H11" s="39" t="inlineStr">
+      <c r="H11" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8153,7 +8153,7 @@
           <t>1-1</t>
         </is>
       </c>
-      <c r="M11" s="39" t="inlineStr">
+      <c r="M11" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8200,7 +8200,7 @@
           <t>4-0</t>
         </is>
       </c>
-      <c r="C12" s="39" t="inlineStr">
+      <c r="C12" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8215,12 +8215,12 @@
           <t>3-3</t>
         </is>
       </c>
-      <c r="F12" s="39" t="inlineStr">
+      <c r="F12" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="G12" s="39" t="inlineStr">
+      <c r="G12" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8260,7 +8260,7 @@
           <t>4-2</t>
         </is>
       </c>
-      <c r="O12" s="39" t="inlineStr">
+      <c r="O12" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8307,7 +8307,7 @@
           <t>2-4</t>
         </is>
       </c>
-      <c r="E13" s="39" t="inlineStr">
+      <c r="E13" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8317,7 +8317,7 @@
           <t>1-0</t>
         </is>
       </c>
-      <c r="G13" s="39" t="inlineStr">
+      <c r="G13" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8337,7 +8337,7 @@
           <t>3-1</t>
         </is>
       </c>
-      <c r="K13" s="39" t="inlineStr">
+      <c r="K13" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8362,7 +8362,7 @@
           <t>2-2</t>
         </is>
       </c>
-      <c r="P13" s="39" t="inlineStr">
+      <c r="P13" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8377,7 +8377,7 @@
           <t>1-3</t>
         </is>
       </c>
-      <c r="S13" s="39" t="inlineStr">
+      <c r="S13" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8404,7 +8404,7 @@
           <t>1-1</t>
         </is>
       </c>
-      <c r="E14" s="39" t="inlineStr">
+      <c r="E14" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8419,7 +8419,7 @@
           <t>1-1</t>
         </is>
       </c>
-      <c r="H14" s="39" t="inlineStr">
+      <c r="H14" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8434,7 +8434,7 @@
           <t>5-0</t>
         </is>
       </c>
-      <c r="K14" s="39" t="inlineStr">
+      <c r="K14" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8449,12 +8449,12 @@
           <t>—</t>
         </is>
       </c>
-      <c r="N14" s="39" t="inlineStr">
+      <c r="N14" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="O14" s="39" t="inlineStr">
+      <c r="O14" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8506,7 +8506,7 @@
           <t>1-1</t>
         </is>
       </c>
-      <c r="F15" s="39" t="inlineStr">
+      <c r="F15" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8521,12 +8521,12 @@
           <t>2-1</t>
         </is>
       </c>
-      <c r="I15" s="39" t="inlineStr">
+      <c r="I15" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="J15" s="39" t="inlineStr">
+      <c r="J15" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8566,7 +8566,7 @@
           <t>1-2</t>
         </is>
       </c>
-      <c r="R15" s="39" t="inlineStr">
+      <c r="R15" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8618,7 +8618,7 @@
           <t>1-2</t>
         </is>
       </c>
-      <c r="I16" s="39" t="inlineStr">
+      <c r="I16" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8633,7 +8633,7 @@
           <t>0-0</t>
         </is>
       </c>
-      <c r="L16" s="39" t="inlineStr">
+      <c r="L16" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8663,12 +8663,12 @@
           <t>2-0</t>
         </is>
       </c>
-      <c r="R16" s="39" t="inlineStr">
+      <c r="R16" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="S16" s="39" t="inlineStr">
+      <c r="S16" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8680,12 +8680,12 @@
           <t>VVV-Venlo</t>
         </is>
       </c>
-      <c r="B17" s="39" t="inlineStr">
+      <c r="B17" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="C17" s="39" t="inlineStr">
+      <c r="C17" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8745,7 +8745,7 @@
           <t>3-1</t>
         </is>
       </c>
-      <c r="O17" s="39" t="inlineStr">
+      <c r="O17" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8760,7 +8760,7 @@
           <t>0-4</t>
         </is>
       </c>
-      <c r="R17" s="39" t="inlineStr">
+      <c r="R17" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8822,7 +8822,7 @@
           <t>4-2</t>
         </is>
       </c>
-      <c r="K18" s="39" t="inlineStr">
+      <c r="K18" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8837,12 +8837,12 @@
           <t>1-2</t>
         </is>
       </c>
-      <c r="N18" s="39" t="inlineStr">
+      <c r="N18" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="O18" s="39" t="inlineStr">
+      <c r="O18" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8857,7 +8857,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="R18" s="39" t="inlineStr">
+      <c r="R18" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8874,7 +8874,7 @@
           <t>Willem II</t>
         </is>
       </c>
-      <c r="B19" s="39" t="inlineStr">
+      <c r="B19" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8884,7 +8884,7 @@
           <t>1-0</t>
         </is>
       </c>
-      <c r="D19" s="39" t="inlineStr">
+      <c r="D19" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8899,7 +8899,7 @@
           <t>3-1</t>
         </is>
       </c>
-      <c r="G19" s="39" t="inlineStr">
+      <c r="G19" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8959,7 +8959,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="S19" s="39" t="inlineStr">
+      <c r="S19" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -8986,7 +8986,7 @@
           <t>1-3</t>
         </is>
       </c>
-      <c r="E20" s="39" t="inlineStr">
+      <c r="E20" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -9026,12 +9026,12 @@
           <t>1-0</t>
         </is>
       </c>
-      <c r="M20" s="39" t="inlineStr">
+      <c r="M20" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
       </c>
-      <c r="N20" s="39" t="inlineStr">
+      <c r="N20" s="41" t="inlineStr">
         <is>
           <t>·</t>
         </is>
@@ -9063,7 +9063,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="40" t="inlineStr">
+      <c r="A22" s="39" t="inlineStr">
         <is>
           <t>🟢 Groen = Thuiswinst   🔴 Rood = Thuisverlies   🟡 Geel = Gelijk   · = Niet gespeeld</t>
         </is>
@@ -11791,7 +11791,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="40" t="inlineStr">
+      <c r="A22" s="39" t="inlineStr">
         <is>
           <t>🟢 Groen = Thuiswinst   🔴 Rood = Thuisverlies   🟡 Geel = Gelijk   · = Niet gespeeld</t>
         </is>
@@ -14519,7 +14519,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="40" t="inlineStr">
+      <c r="A22" s="39" t="inlineStr">
         <is>
           <t>🟢 Groen = Thuiswinst   🔴 Rood = Thuisverlies   🟡 Geel = Gelijk   · = Niet gespeeld</t>
         </is>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  26 May 2026 om 18:06</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  27 May 2026 om 18:07</t>
         </is>
       </c>
     </row>
@@ -16551,9 +16551,9 @@
           <t>0-2</t>
         </is>
       </c>
-      <c r="Q13" s="39" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="Q13" s="36" t="inlineStr">
+        <is>
+          <t>2-0</t>
         </is>
       </c>
       <c r="R13" s="37" t="inlineStr">
@@ -17247,7 +17247,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="40" t="inlineStr">
+      <c r="A22" s="39" t="inlineStr">
         <is>
           <t>🟢 Groen = Thuiswinst   🔴 Rood = Thuisverlies   🟡 Geel = Gelijk   · = Nog niet gespeeld</t>
         </is>
@@ -19143,7 +19143,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="40" t="inlineStr">
+      <c r="A22" s="39" t="inlineStr">
         <is>
           <t>🟢 Groen = Thuiswinst   🔴 Rood = Thuisverlies   🟡 Geel = Gelijk   · = Niet gespeeld</t>
         </is>
@@ -19479,7 +19479,7 @@
       <c r="I8" s="10" t="n">
         <v>49</v>
       </c>
-      <c r="J8" s="41" t="inlineStr">
+      <c r="J8" s="40" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -21871,7 +21871,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="40" t="inlineStr">
+      <c r="A22" s="39" t="inlineStr">
         <is>
           <t>🟢 Groen = Thuiswinst   🔴 Rood = Thuisverlies   🟡 Geel = Gelijk   · = Niet gespeeld</t>
         </is>
@@ -24599,7 +24599,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="40" t="inlineStr">
+      <c r="A22" s="39" t="inlineStr">
         <is>
           <t>🟢 Groen = Thuiswinst   🔴 Rood = Thuisverlies   🟡 Geel = Gelijk   · = Niet gespeeld</t>
         </is>
@@ -27327,7 +27327,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="40" t="inlineStr">
+      <c r="A22" s="39" t="inlineStr">
         <is>
           <t>🟢 Groen = Thuiswinst   🔴 Rood = Thuisverlies   🟡 Geel = Gelijk   · = Niet gespeeld</t>
         </is>
@@ -30055,7 +30055,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="40" t="inlineStr">
+      <c r="A22" s="39" t="inlineStr">
         <is>
           <t>🟢 Groen = Thuiswinst   🔴 Rood = Thuisverlies   🟡 Geel = Gelijk   · = Niet gespeeld</t>
         </is>
@@ -33615,7 +33615,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="40" t="inlineStr">
+      <c r="A22" s="39" t="inlineStr">
         <is>
           <t>🟢 Groen = Thuiswinst   🔴 Rood = Thuisverlies   🟡 Geel = Gelijk   · = Niet gespeeld</t>
         </is>
@@ -36290,7 +36290,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="40" t="inlineStr">
+      <c r="A22" s="39" t="inlineStr">
         <is>
           <t>🟢 Groen = Thuiswinst   🔴 Rood = Thuisverlies   🟡 Geel = Gelijk   · = Niet gespeeld</t>
         </is>
@@ -39018,7 +39018,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="40" t="inlineStr">
+      <c r="A22" s="39" t="inlineStr">
         <is>
           <t>🟢 Groen = Thuiswinst   🔴 Rood = Thuisverlies   🟡 Geel = Gelijk   · = Niet gespeeld</t>
         </is>
@@ -41746,7 +41746,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="40" t="inlineStr">
+      <c r="A22" s="39" t="inlineStr">
         <is>
           <t>🟢 Groen = Thuiswinst   🔴 Rood = Thuisverlies   🟡 Geel = Gelijk   · = Niet gespeeld</t>
         </is>
@@ -42082,7 +42082,7 @@
       <c r="I8" s="10" t="n">
         <v>51</v>
       </c>
-      <c r="J8" s="41" t="inlineStr">
+      <c r="J8" s="40" t="inlineStr">
         <is>
           <t>-9</t>
         </is>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 28-05-2026 18:21
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  27 May 2026 om 18:07</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  28 May 2026 om 18:21</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  27 May 2026 om 18:07</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  28 May 2026 om 18:21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 29-05-2026 18:16
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  28 May 2026 om 18:21</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  29 May 2026 om 18:16</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  28 May 2026 om 18:21</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  29 May 2026 om 18:16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 30-05-2026 11:56
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  29 May 2026 om 18:16</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  30 May 2026 om 11:56</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  29 May 2026 om 18:16</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  30 May 2026 om 11:56</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 31-05-2026 12:03
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  30 May 2026 om 11:56</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  31 May 2026 om 12:03</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  30 May 2026 om 11:56</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  31 May 2026 om 12:03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 01-06-2026 12:41
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  31 May 2026 om 12:03</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  1 June 2026 om 12:41</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  31 May 2026 om 12:03</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  1 June 2026 om 12:41</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 02-06-2026 11:20
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  1 June 2026 om 12:41</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  2 June 2026 om 11:20</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  1 June 2026 om 12:41</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  2 June 2026 om 11:20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 03-06-2026 11:58
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  2 June 2026 om 11:20</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  3 June 2026 om 11:58</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  2 June 2026 om 11:20</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  3 June 2026 om 11:58</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 04-06-2026 10:40
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  3 June 2026 om 11:58</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  4 June 2026 om 10:40</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  3 June 2026 om 11:58</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  4 June 2026 om 10:40</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 05-06-2026 10:50
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  4 June 2026 om 10:40</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  5 June 2026 om 10:50</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  4 June 2026 om 10:40</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  5 June 2026 om 10:50</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 06-06-2026 09:27
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  5 June 2026 om 10:50</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  6 June 2026 om 09:27</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  5 June 2026 om 10:50</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  6 June 2026 om 09:27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 07-06-2026 10:06
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  6 June 2026 om 09:27</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  7 June 2026 om 10:06</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  6 June 2026 om 09:27</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  7 June 2026 om 10:06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 08-06-2026 12:01
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  7 June 2026 om 10:06</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  8 June 2026 om 12:01</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  7 June 2026 om 10:06</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  8 June 2026 om 12:01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 09-06-2026 10:36
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  8 June 2026 om 12:01</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  9 June 2026 om 10:36</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  8 June 2026 om 12:01</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  9 June 2026 om 10:36</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 10-06-2026 10:58
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  9 June 2026 om 10:36</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  10 June 2026 om 10:58</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  9 June 2026 om 10:36</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  10 June 2026 om 10:58</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 11-06-2026 11:24
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  10 June 2026 om 10:58</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  11 June 2026 om 11:24</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  10 June 2026 om 10:58</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  11 June 2026 om 11:24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 12-06-2026 11:03
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  11 June 2026 om 11:24</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  12 June 2026 om 11:03</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  11 June 2026 om 11:24</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  12 June 2026 om 11:03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 13-06-2026 09:57
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  12 June 2026 om 11:03</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  13 June 2026 om 09:57</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  12 June 2026 om 11:03</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  13 June 2026 om 09:57</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 15-06-2026 13:19
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  14 June 2026 om 10:26</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  15 June 2026 om 13:19</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  14 June 2026 om 10:26</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  15 June 2026 om 13:19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 16-06-2026 12:13
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  15 June 2026 om 13:19</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  16 June 2026 om 12:13</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  15 June 2026 om 13:19</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  16 June 2026 om 12:13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 17-06-2026 11:51
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  16 June 2026 om 12:13</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  17 June 2026 om 11:51</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  16 June 2026 om 12:13</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  17 June 2026 om 11:51</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 18-06-2026 11:09
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  17 June 2026 om 11:51</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  18 June 2026 om 11:09</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  17 June 2026 om 11:51</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  18 June 2026 om 11:09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 19-06-2026 11:25
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  18 June 2026 om 11:09</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  19 June 2026 om 11:25</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  18 June 2026 om 11:09</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  19 June 2026 om 11:25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 20-06-2026 10:10
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  19 June 2026 om 11:25</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  20 June 2026 om 10:10</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  19 June 2026 om 11:25</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  20 June 2026 om 10:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 21-06-2026 10:32
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  20 June 2026 om 10:10</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  21 June 2026 om 10:32</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  20 June 2026 om 10:10</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  21 June 2026 om 10:32</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 22-06-2026 12:51
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  21 June 2026 om 10:32</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  22 June 2026 om 12:51</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  21 June 2026 om 10:32</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  22 June 2026 om 12:51</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 23-06-2026 10:37
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  22 June 2026 om 12:51</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  23 June 2026 om 10:37</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  22 June 2026 om 12:51</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  23 June 2026 om 10:37</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 24-06-2026 10:24
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  23 June 2026 om 10:37</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  24 June 2026 om 10:24</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  23 June 2026 om 10:37</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  24 June 2026 om 10:24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 25-06-2026 10:16
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  24 June 2026 om 10:24</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  25 June 2026 om 10:16</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  24 June 2026 om 10:24</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  25 June 2026 om 10:16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 26-06-2026 10:24
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  25 June 2026 om 10:16</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  26 June 2026 om 10:24</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  25 June 2026 om 10:16</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  26 June 2026 om 10:24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 27-06-2026 09:30
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  26 June 2026 om 10:24</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  27 June 2026 om 09:30</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  26 June 2026 om 10:24</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  27 June 2026 om 09:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 28-06-2026 10:05
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  27 June 2026 om 09:30</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  28 June 2026 om 10:05</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  27 June 2026 om 09:30</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  28 June 2026 om 10:05</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 29-06-2026 12:01
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  28 June 2026 om 10:05</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  29 June 2026 om 12:01</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  28 June 2026 om 10:05</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  29 June 2026 om 12:01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 30-06-2026 10:32
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  29 June 2026 om 12:01</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  30 June 2026 om 10:32</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  29 June 2026 om 12:01</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  30 June 2026 om 10:32</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 01-07-2026 10:43
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  30 June 2026 om 10:32</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  1 July 2026 om 10:43</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  30 June 2026 om 10:32</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  1 July 2026 om 10:43</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 02-07-2026 10:11
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  1 July 2026 om 10:43</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  2 July 2026 om 10:11</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  1 July 2026 om 10:43</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  2 July 2026 om 10:11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 03-07-2026 10:07
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  2 July 2026 om 10:11</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  3 July 2026 om 10:07</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  2 July 2026 om 10:11</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  3 July 2026 om 10:07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 04-07-2026 09:24
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  3 July 2026 om 10:07</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  4 July 2026 om 09:24</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  3 July 2026 om 10:07</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  4 July 2026 om 09:24</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 05-07-2026 09:43
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  4 July 2026 om 09:24</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  5 July 2026 om 09:43</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  4 July 2026 om 09:24</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  5 July 2026 om 09:43</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 06-07-2026 11:39
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  5 July 2026 om 09:43</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  6 July 2026 om 11:39</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  5 July 2026 om 09:43</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  6 July 2026 om 11:39</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 07-07-2026 10:27
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  6 July 2026 om 11:39</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  7 July 2026 om 10:27</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  6 July 2026 om 11:39</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  7 July 2026 om 10:27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 08-07-2026 09:27
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  7 July 2026 om 10:27</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  8 July 2026 om 09:27</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  7 July 2026 om 10:27</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  8 July 2026 om 09:27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 09-07-2026 10:26
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  8 July 2026 om 09:27</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  9 July 2026 om 10:26</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  8 July 2026 om 09:27</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  9 July 2026 om 10:26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 10-07-2026 10:25
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  9 July 2026 om 10:26</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  10 July 2026 om 10:25</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  9 July 2026 om 10:26</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  10 July 2026 om 10:25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 11-07-2026 08:49
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  10 July 2026 om 10:25</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  11 July 2026 om 08:49</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  10 July 2026 om 10:25</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  11 July 2026 om 08:49</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 12-07-2026 09:05
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  11 July 2026 om 08:49</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  12 July 2026 om 09:04</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  11 July 2026 om 08:49</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  12 July 2026 om 09:04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 13-07-2026 10:29
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  12 July 2026 om 09:04</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  13 July 2026 om 10:29</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  12 July 2026 om 09:04</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  13 July 2026 om 10:29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 14-07-2026 09:06
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  13 July 2026 om 10:29</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  14 July 2026 om 09:06</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  13 July 2026 om 10:29</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  14 July 2026 om 09:06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 15-07-2026 09:10
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  14 July 2026 om 09:06</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  15 July 2026 om 09:10</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  14 July 2026 om 09:06</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  15 July 2026 om 09:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 16-07-2026 09:17
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  15 July 2026 om 09:10</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  16 July 2026 om 09:17</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  15 July 2026 om 09:10</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  16 July 2026 om 09:17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 17-07-2026 09:11
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  16 July 2026 om 09:17</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  17 July 2026 om 09:11</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  16 July 2026 om 09:17</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  17 July 2026 om 09:11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 18-07-2026 08:49
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  17 July 2026 om 09:11</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  18 July 2026 om 08:49</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  17 July 2026 om 09:11</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  18 July 2026 om 08:49</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 19-07-2026 09:06
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  18 July 2026 om 08:49</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  19 July 2026 om 09:06</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  18 July 2026 om 08:49</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  19 July 2026 om 09:06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 20-07-2026 10:14
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  19 July 2026 om 09:06</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  20 July 2026 om 10:14</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  19 July 2026 om 09:06</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  20 July 2026 om 10:14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 21-07-2026 09:29
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  20 July 2026 om 10:14</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  21 July 2026 om 09:29</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  20 July 2026 om 10:14</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  21 July 2026 om 09:29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 22-07-2026 09:28
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  21 July 2026 om 09:29</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  22 July 2026 om 09:28</t>
         </is>
       </c>
     </row>
@@ -986,7 +986,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>ADO Den Haag</t>
+          <t>Telstar 1963</t>
         </is>
       </c>
       <c r="C3" s="5" t="n">
@@ -1027,7 +1027,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>AFC Ajax</t>
+          <t>SBV Excelsior</t>
         </is>
       </c>
       <c r="C4" s="5" t="n">
@@ -1068,7 +1068,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>Feyenoord Rotterdam</t>
         </is>
       </c>
       <c r="C5" s="5" t="n">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>FC Twente '65</t>
+          <t>PEC Zwolle</t>
         </is>
       </c>
       <c r="C7" s="5" t="n">
@@ -1191,7 +1191,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>FC Utrecht</t>
+          <t>FC Twente '65</t>
         </is>
       </c>
       <c r="C8" s="5" t="n">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Feyenoord Rotterdam</t>
+          <t>SC Cambuur-Leeuwarden</t>
         </is>
       </c>
       <c r="C9" s="5" t="n">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Fortuna Sittard</t>
+          <t>AFC Ajax</t>
         </is>
       </c>
       <c r="C10" s="5" t="n">
@@ -1314,7 +1314,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Go Ahead Eagles</t>
+          <t>NEC</t>
         </is>
       </c>
       <c r="C11" s="5" t="n">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>NEC</t>
+          <t>FC Utrecht</t>
         </is>
       </c>
       <c r="C12" s="5" t="n">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>PEC Zwolle</t>
+          <t>Sparta Rotterdam</t>
         </is>
       </c>
       <c r="C13" s="5" t="n">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>PSV</t>
+          <t>Fortuna Sittard</t>
         </is>
       </c>
       <c r="C14" s="5" t="n">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>SBV Excelsior</t>
+          <t>SC Heerenveen</t>
         </is>
       </c>
       <c r="C15" s="5" t="n">
@@ -1519,7 +1519,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>SC Cambuur-Leeuwarden</t>
+          <t>PSV</t>
         </is>
       </c>
       <c r="C16" s="5" t="n">
@@ -1560,7 +1560,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>SC Heerenveen</t>
+          <t>Willem II Tilburg</t>
         </is>
       </c>
       <c r="C17" s="5" t="n">
@@ -1601,7 +1601,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Sparta Rotterdam</t>
+          <t>Go Ahead Eagles</t>
         </is>
       </c>
       <c r="C18" s="5" t="n">
@@ -1642,7 +1642,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Telstar 1963</t>
+          <t>ADO Den Haag</t>
         </is>
       </c>
       <c r="C19" s="5" t="n">
@@ -1683,7 +1683,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Willem II Tilburg</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="C20" s="5" t="n">
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  21 July 2026 om 09:29</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  22 July 2026 om 09:28</t>
         </is>
       </c>
     </row>
@@ -33725,7 +33725,7 @@
       </c>
       <c r="B5" s="45" t="inlineStr">
         <is>
-          <t>ADO Den Haag</t>
+          <t>Telstar 1963</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
@@ -33855,14 +33855,14 @@
       </c>
       <c r="H8" s="48" t="inlineStr">
         <is>
-          <t>ADO Den Haag</t>
+          <t>Telstar 1963</t>
         </is>
       </c>
       <c r="I8" s="26" t="n">
         <v>1</v>
       </c>
       <c r="J8" s="28" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1">

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 23-07-2026 09:26
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  22 July 2026 om 09:28</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  23 July 2026 om 09:26</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  22 July 2026 om 09:28</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  23 July 2026 om 09:26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 24-07-2026 09:22
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  23 July 2026 om 09:26</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  24 July 2026 om 09:22</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  23 July 2026 om 09:26</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  24 July 2026 om 09:22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 25-07-2026 09:01
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  24 July 2026 om 09:22</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  25 July 2026 om 09:01</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  24 July 2026 om 09:22</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  25 July 2026 om 09:01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 26-07-2026 09:16
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  25 July 2026 om 09:01</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  26 July 2026 om 09:16</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  25 July 2026 om 09:01</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  26 July 2026 om 09:16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 27-07-2026 10:45
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  26 July 2026 om 09:16</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  27 July 2026 om 10:45</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  26 July 2026 om 09:16</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  27 July 2026 om 10:45</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 28-07-2026 09:37
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  27 July 2026 om 10:45</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  28 July 2026 om 09:37</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  27 July 2026 om 10:45</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  28 July 2026 om 09:37</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 29-07-2026 09:39
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  28 July 2026 om 09:37</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  29 July 2026 om 09:39</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  28 July 2026 om 09:37</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  29 July 2026 om 09:39</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 30-07-2026 09:33
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  29 July 2026 om 09:39</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  30 July 2026 om 09:33</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  29 July 2026 om 09:39</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  30 July 2026 om 09:33</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 31-07-2026 09:47
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  30 July 2026 om 09:33</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  31 July 2026 om 09:47</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  30 July 2026 om 09:33</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  31 July 2026 om 09:47</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 01-08-2026 09:07
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  31 July 2026 om 09:47</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  1 August 2026 om 09:07</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  31 July 2026 om 09:47</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  1 August 2026 om 09:07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 02-08-2026 09:11
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  1 August 2026 om 09:07</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  2 August 2026 om 09:11</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  1 August 2026 om 09:07</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  2 August 2026 om 09:11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 03-08-2026 10:45
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  2 August 2026 om 09:11</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  3 August 2026 om 10:45</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  2 August 2026 om 09:11</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  3 August 2026 om 10:45</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 04-08-2026 09:39
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  3 August 2026 om 10:45</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  4 August 2026 om 09:39</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  3 August 2026 om 10:45</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  4 August 2026 om 09:39</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 05-08-2026 09:38
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  4 August 2026 om 09:39</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  5 August 2026 om 09:38</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  4 August 2026 om 09:39</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  5 August 2026 om 09:38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 06-08-2026 09:41
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  5 August 2026 om 09:38</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  6 August 2026 om 09:41</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  5 August 2026 om 09:38</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  6 August 2026 om 09:41</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 07-08-2026 08:16
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  6 August 2026 om 09:41</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  7 August 2026 om 08:16</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  6 August 2026 om 09:41</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  7 August 2026 om 08:16</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 11-08-2026 08:10
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  10 August 2026 om 08:41</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  11 August 2026 om 08:10</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  10 August 2026 om 08:41</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  11 August 2026 om 08:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 12-08-2026 08:20
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  11 August 2026 om 08:10</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  12 August 2026 om 08:20</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  11 August 2026 om 08:10</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  12 August 2026 om 08:20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 13-08-2026 08:23
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  12 August 2026 om 08:20</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  13 August 2026 om 08:23</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  12 August 2026 om 08:20</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  13 August 2026 om 08:23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 14-08-2026 08:18
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  13 August 2026 om 08:23</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  14 August 2026 om 08:18</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  13 August 2026 om 08:23</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  14 August 2026 om 08:18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 15-08-2026 07:33
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  14 August 2026 om 08:18</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  15 August 2026 om 07:33</t>
         </is>
       </c>
     </row>
@@ -1150,11 +1150,11 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>FC Groningen</t>
+          <t>Sparta Rotterdam</t>
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7" s="10" t="n">
         <v>1</v>
@@ -1163,17 +1163,17 @@
         <v>0</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" s="11" t="n">
         <v>3</v>
       </c>
       <c r="H7" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="I7" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="I7" s="10" t="n">
-        <v>1</v>
-      </c>
       <c r="J7" s="12" t="inlineStr">
         <is>
           <t>+1</t>
@@ -1181,17 +1181,17 @@
       </c>
       <c r="K7" s="10" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>50%</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Telstar 1963</t>
+          <t>FC Groningen</t>
         </is>
       </c>
       <c r="C8" s="10" t="n">
@@ -1314,48 +1314,48 @@
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>Fortuna Sittard</t>
+          <t>Telstar 1963</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="15" t="n">
+      <c r="E11" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="15" t="n">
+      <c r="F11" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="F11" s="15" t="n">
-        <v>0</v>
-      </c>
       <c r="G11" s="16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I11" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="J11" s="15" t="inlineStr">
-        <is>
-          <t>0</t>
+        <v>4</v>
+      </c>
+      <c r="J11" s="23" t="inlineStr">
+        <is>
+          <t>-1</t>
         </is>
       </c>
       <c r="K11" s="15" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>50%</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="18" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>PSV</t>
+          <t>Fortuna Sittard</t>
         </is>
       </c>
       <c r="C12" s="20" t="n">
@@ -1392,11 +1392,11 @@
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="13" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>FC Utrecht</t>
+          <t>PSV</t>
         </is>
       </c>
       <c r="C13" s="15" t="n">
@@ -1406,23 +1406,23 @@
         <v>0</v>
       </c>
       <c r="E13" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="15" t="n">
+      <c r="G13" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="G13" s="16" t="n">
-        <v>0</v>
-      </c>
       <c r="H13" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I13" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
-        <is>
-          <t>-1</t>
+      <c r="J13" s="15" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
       <c r="K13" s="15" t="inlineStr">
@@ -1433,11 +1433,11 @@
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="18" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B14" s="19" t="inlineStr">
         <is>
-          <t>NEC</t>
+          <t>FC Utrecht</t>
         </is>
       </c>
       <c r="C14" s="20" t="n">
@@ -1474,11 +1474,11 @@
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="13" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>FC Twente '65</t>
+          <t>NEC</t>
         </is>
       </c>
       <c r="C15" s="15" t="n">
@@ -1497,10 +1497,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I15" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J15" s="23" t="inlineStr">
         <is>
@@ -1515,11 +1515,11 @@
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="18" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>Sparta Rotterdam</t>
+          <t>FC Twente '65</t>
         </is>
       </c>
       <c r="C16" s="20" t="n">
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  14 August 2026 om 08:18</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  15 August 2026 om 07:33</t>
         </is>
       </c>
     </row>
@@ -17133,9 +17133,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="Q19" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="Q19" s="38" t="inlineStr">
+        <is>
+          <t>1-3</t>
         </is>
       </c>
       <c r="R19" s="34" t="inlineStr">

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 16-08-2026 07:33
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -333,10 +333,10 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  15 August 2026 om 07:33</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  16 August 2026 om 07:33</t>
         </is>
       </c>
     </row>
@@ -986,14 +986,14 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>SBV Excelsior</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="C3" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>0</v>
@@ -1002,17 +1002,17 @@
         <v>0</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>+4</t>
+          <t>+5</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
@@ -1027,38 +1027,38 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Go Ahead Eagles</t>
+          <t>Fortuna Sittard</t>
         </is>
       </c>
       <c r="C4" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E4" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" s="10" t="n">
         <v>0</v>
       </c>
       <c r="G4" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H4" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="I4" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="H4" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="I4" s="10" t="n">
-        <v>1</v>
-      </c>
       <c r="J4" s="12" t="inlineStr">
         <is>
-          <t>+3</t>
+          <t>+2</t>
         </is>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>50%</t>
         </is>
       </c>
     </row>
@@ -1068,52 +1068,52 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>AFC Ajax</t>
+          <t>PSV</t>
         </is>
       </c>
       <c r="C5" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E5" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" s="10" t="n">
         <v>0</v>
       </c>
       <c r="G5" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H5" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="I5" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="H5" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="I5" s="10" t="n">
-        <v>0</v>
-      </c>
       <c r="J5" s="12" t="inlineStr">
         <is>
-          <t>+2</t>
+          <t>+1</t>
         </is>
       </c>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>50%</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>SBV Excelsior</t>
         </is>
       </c>
       <c r="C6" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D6" s="10" t="n">
         <v>1</v>
@@ -1122,25 +1122,25 @@
         <v>0</v>
       </c>
       <c r="F6" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G6" s="11" t="n">
         <v>3</v>
       </c>
       <c r="H6" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="I6" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="I6" s="10" t="n">
-        <v>0</v>
-      </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
-          <t>+2</t>
+          <t>+3</t>
         </is>
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>50%</t>
         </is>
       </c>
     </row>
@@ -1150,11 +1150,11 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Sparta Rotterdam</t>
+          <t>Go Ahead Eagles</t>
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D7" s="10" t="n">
         <v>1</v>
@@ -1163,25 +1163,25 @@
         <v>0</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7" s="11" t="n">
         <v>3</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J7" s="12" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>+3</t>
         </is>
       </c>
       <c r="K7" s="10" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>100%</t>
         </is>
       </c>
     </row>
@@ -1191,11 +1191,11 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>FC Groningen</t>
+          <t>NEC</t>
         </is>
       </c>
       <c r="C8" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" s="10" t="n">
         <v>1</v>
@@ -1204,25 +1204,25 @@
         <v>0</v>
       </c>
       <c r="F8" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" s="11" t="n">
         <v>3</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J8" s="12" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>+2</t>
         </is>
       </c>
       <c r="K8" s="10" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>50%</t>
         </is>
       </c>
     </row>
@@ -1232,7 +1232,7 @@
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>Feyenoord Rotterdam</t>
+          <t>AFC Ajax</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
@@ -1251,14 +1251,14 @@
         <v>3</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I9" s="15" t="n">
         <v>0</v>
       </c>
       <c r="J9" s="17" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>+2</t>
         </is>
       </c>
       <c r="K9" s="15" t="inlineStr">
@@ -1269,15 +1269,15 @@
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="18" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>SC Heerenveen</t>
+          <t>Sparta Rotterdam</t>
         </is>
       </c>
       <c r="C10" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D10" s="20" t="n">
         <v>1</v>
@@ -1286,16 +1286,16 @@
         <v>0</v>
       </c>
       <c r="F10" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" s="21" t="n">
         <v>3</v>
       </c>
       <c r="H10" s="20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I10" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J10" s="22" t="inlineStr">
         <is>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="K10" s="20" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>50%</t>
         </is>
       </c>
     </row>
@@ -1314,11 +1314,11 @@
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>Telstar 1963</t>
+          <t>FC Groningen</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D11" s="15" t="n">
         <v>1</v>
@@ -1327,25 +1327,25 @@
         <v>0</v>
       </c>
       <c r="F11" s="15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" s="16" t="n">
         <v>3</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I11" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="J11" s="23" t="inlineStr">
-        <is>
-          <t>-1</t>
+        <v>1</v>
+      </c>
+      <c r="J11" s="17" t="inlineStr">
+        <is>
+          <t>+1</t>
         </is>
       </c>
       <c r="K11" s="15" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>100%</t>
         </is>
       </c>
     </row>
@@ -1355,38 +1355,38 @@
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>Fortuna Sittard</t>
+          <t>Feyenoord Rotterdam</t>
         </is>
       </c>
       <c r="C12" s="20" t="n">
         <v>1</v>
       </c>
       <c r="D12" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="20" t="n">
         <v>0</v>
-      </c>
-      <c r="E12" s="20" t="n">
-        <v>1</v>
       </c>
       <c r="F12" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G12" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="H12" s="20" t="n">
-        <v>2</v>
-      </c>
       <c r="I12" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="J12" s="20" t="inlineStr">
-        <is>
-          <t>0</t>
+        <v>0</v>
+      </c>
+      <c r="J12" s="22" t="inlineStr">
+        <is>
+          <t>+1</t>
         </is>
       </c>
       <c r="K12" s="20" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
     </row>
@@ -1396,38 +1396,38 @@
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>PSV</t>
+          <t>SC Heerenveen</t>
         </is>
       </c>
       <c r="C13" s="15" t="n">
         <v>1</v>
       </c>
       <c r="D13" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="15" t="n">
         <v>0</v>
-      </c>
-      <c r="E13" s="15" t="n">
-        <v>1</v>
       </c>
       <c r="F13" s="15" t="n">
         <v>0</v>
       </c>
       <c r="G13" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="H13" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="H13" s="15" t="n">
-        <v>2</v>
-      </c>
       <c r="I13" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="J13" s="15" t="inlineStr">
-        <is>
-          <t>0</t>
+        <v>0</v>
+      </c>
+      <c r="J13" s="17" t="inlineStr">
+        <is>
+          <t>+1</t>
         </is>
       </c>
       <c r="K13" s="15" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
     </row>
@@ -1437,14 +1437,14 @@
       </c>
       <c r="B14" s="19" t="inlineStr">
         <is>
-          <t>FC Utrecht</t>
+          <t>Telstar 1963</t>
         </is>
       </c>
       <c r="C14" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="20" t="n">
         <v>1</v>
-      </c>
-      <c r="D14" s="20" t="n">
-        <v>0</v>
       </c>
       <c r="E14" s="20" t="n">
         <v>0</v>
@@ -1453,32 +1453,32 @@
         <v>1</v>
       </c>
       <c r="G14" s="21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H14" s="20" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I14" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="J14" s="24" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-1</t>
         </is>
       </c>
       <c r="K14" s="20" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>50%</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>NEC</t>
+          <t>FC Twente '65</t>
         </is>
       </c>
       <c r="C15" s="15" t="n">
@@ -1497,12 +1497,12 @@
         <v>0</v>
       </c>
       <c r="H15" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="I15" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-1</t>
         </is>
@@ -1519,7 +1519,7 @@
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>FC Twente '65</t>
+          <t>ADO Den Haag</t>
         </is>
       </c>
       <c r="C16" s="20" t="n">
@@ -1541,11 +1541,11 @@
         <v>0</v>
       </c>
       <c r="I16" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="J16" s="24" t="inlineStr">
-        <is>
-          <t>-1</t>
+        <v>2</v>
+      </c>
+      <c r="J16" s="23" t="inlineStr">
+        <is>
+          <t>-2</t>
         </is>
       </c>
       <c r="K16" s="20" t="inlineStr">
@@ -1556,11 +1556,11 @@
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="13" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>ADO Den Haag</t>
+          <t>PEC Zwolle</t>
         </is>
       </c>
       <c r="C17" s="15" t="n">
@@ -1584,7 +1584,7 @@
       <c r="I17" s="15" t="n">
         <v>2</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -1597,15 +1597,15 @@
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="18" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>PEC Zwolle</t>
+          <t>FC Utrecht</t>
         </is>
       </c>
       <c r="C18" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" s="20" t="n">
         <v>0</v>
@@ -1614,20 +1614,20 @@
         <v>0</v>
       </c>
       <c r="F18" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G18" s="21" t="n">
         <v>0</v>
       </c>
       <c r="H18" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I18" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="J18" s="24" t="inlineStr">
-        <is>
-          <t>-2</t>
+        <v>6</v>
+      </c>
+      <c r="J18" s="23" t="inlineStr">
+        <is>
+          <t>-4</t>
         </is>
       </c>
       <c r="K18" s="20" t="inlineStr">
@@ -1646,7 +1646,7 @@
         </is>
       </c>
       <c r="C19" s="27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D19" s="27" t="n">
         <v>0</v>
@@ -1655,20 +1655,20 @@
         <v>0</v>
       </c>
       <c r="F19" s="27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G19" s="28" t="n">
         <v>0</v>
       </c>
       <c r="H19" s="27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I19" s="27" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J19" s="29" t="inlineStr">
         <is>
-          <t>-3</t>
+          <t>-6</t>
         </is>
       </c>
       <c r="K19" s="27" t="inlineStr">
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="C20" s="27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D20" s="27" t="n">
         <v>0</v>
@@ -1696,20 +1696,20 @@
         <v>0</v>
       </c>
       <c r="F20" s="27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G20" s="28" t="n">
         <v>0</v>
       </c>
       <c r="H20" s="27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I20" s="27" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J20" s="29" t="inlineStr">
         <is>
-          <t>-4</t>
+          <t>-6</t>
         </is>
       </c>
       <c r="K20" s="27" t="inlineStr">
@@ -4066,7 +4066,7 @@
       <c r="I11" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="24" t="inlineStr">
         <is>
           <t>-11</t>
         </is>
@@ -4107,7 +4107,7 @@
       <c r="I12" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J12" s="24" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -4148,7 +4148,7 @@
       <c r="I13" s="15" t="n">
         <v>58</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-8</t>
         </is>
@@ -4189,7 +4189,7 @@
       <c r="I14" s="20" t="n">
         <v>49</v>
       </c>
-      <c r="J14" s="24" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-6</t>
         </is>
@@ -4230,7 +4230,7 @@
       <c r="I15" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -4271,7 +4271,7 @@
       <c r="I16" s="20" t="n">
         <v>68</v>
       </c>
-      <c r="J16" s="24" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-28</t>
         </is>
@@ -4312,7 +4312,7 @@
       <c r="I17" s="15" t="n">
         <v>55</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -4353,7 +4353,7 @@
       <c r="I18" s="20" t="n">
         <v>68</v>
       </c>
-      <c r="J18" s="24" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-28</t>
         </is>
@@ -6794,7 +6794,7 @@
       <c r="I11" s="15" t="n">
         <v>41</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="24" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
@@ -6835,7 +6835,7 @@
       <c r="I12" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="J12" s="24" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
@@ -6917,7 +6917,7 @@
       <c r="I14" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="J14" s="24" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -6958,7 +6958,7 @@
       <c r="I15" s="15" t="n">
         <v>55</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -6999,7 +6999,7 @@
       <c r="I16" s="20" t="n">
         <v>52</v>
       </c>
-      <c r="J16" s="24" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-23</t>
         </is>
@@ -7040,7 +7040,7 @@
       <c r="I17" s="15" t="n">
         <v>51</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-27</t>
         </is>
@@ -7081,7 +7081,7 @@
       <c r="I18" s="20" t="n">
         <v>46</v>
       </c>
-      <c r="J18" s="24" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-12</t>
         </is>
@@ -9440,7 +9440,7 @@
       <c r="I9" s="15" t="n">
         <v>68</v>
       </c>
-      <c r="J9" s="23" t="inlineStr">
+      <c r="J9" s="24" t="inlineStr">
         <is>
           <t>-7</t>
         </is>
@@ -9481,7 +9481,7 @@
       <c r="I10" s="20" t="n">
         <v>41</v>
       </c>
-      <c r="J10" s="24" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -9522,7 +9522,7 @@
       <c r="I11" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="24" t="inlineStr">
         <is>
           <t>-5</t>
         </is>
@@ -9563,7 +9563,7 @@
       <c r="I12" s="20" t="n">
         <v>72</v>
       </c>
-      <c r="J12" s="24" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -9604,7 +9604,7 @@
       <c r="I13" s="15" t="n">
         <v>73</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -9645,7 +9645,7 @@
       <c r="I14" s="20" t="n">
         <v>63</v>
       </c>
-      <c r="J14" s="24" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-16</t>
         </is>
@@ -9686,7 +9686,7 @@
       <c r="I15" s="15" t="n">
         <v>57</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -9727,7 +9727,7 @@
       <c r="I16" s="20" t="n">
         <v>72</v>
       </c>
-      <c r="J16" s="24" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-31</t>
         </is>
@@ -9768,7 +9768,7 @@
       <c r="I17" s="15" t="n">
         <v>80</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-30</t>
         </is>
@@ -9809,7 +9809,7 @@
       <c r="I18" s="20" t="n">
         <v>79</v>
       </c>
-      <c r="J18" s="24" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-33</t>
         </is>
@@ -12168,7 +12168,7 @@
       <c r="I9" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J9" s="23" t="inlineStr">
+      <c r="J9" s="24" t="inlineStr">
         <is>
           <t>-8</t>
         </is>
@@ -12209,7 +12209,7 @@
       <c r="I10" s="20" t="n">
         <v>53</v>
       </c>
-      <c r="J10" s="24" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>-5</t>
         </is>
@@ -12250,7 +12250,7 @@
       <c r="I11" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="24" t="inlineStr">
         <is>
           <t>-12</t>
         </is>
@@ -12291,7 +12291,7 @@
       <c r="I12" s="20" t="n">
         <v>64</v>
       </c>
-      <c r="J12" s="24" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -12332,7 +12332,7 @@
       <c r="I13" s="15" t="n">
         <v>56</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -12414,7 +12414,7 @@
       <c r="I15" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -12455,7 +12455,7 @@
       <c r="I16" s="20" t="n">
         <v>57</v>
       </c>
-      <c r="J16" s="24" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-16</t>
         </is>
@@ -12496,7 +12496,7 @@
       <c r="I17" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -12537,7 +12537,7 @@
       <c r="I18" s="20" t="n">
         <v>69</v>
       </c>
-      <c r="J18" s="24" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-27</t>
         </is>
@@ -14896,7 +14896,7 @@
       <c r="I9" s="15" t="n">
         <v>50</v>
       </c>
-      <c r="J9" s="23" t="inlineStr">
+      <c r="J9" s="24" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -15019,7 +15019,7 @@
       <c r="I12" s="20" t="n">
         <v>55</v>
       </c>
-      <c r="J12" s="24" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -15060,7 +15060,7 @@
       <c r="I13" s="15" t="n">
         <v>59</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -15101,7 +15101,7 @@
       <c r="I14" s="20" t="n">
         <v>60</v>
       </c>
-      <c r="J14" s="24" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -15142,7 +15142,7 @@
       <c r="I15" s="15" t="n">
         <v>44</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -15183,7 +15183,7 @@
       <c r="I16" s="20" t="n">
         <v>67</v>
       </c>
-      <c r="J16" s="24" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-28</t>
         </is>
@@ -15224,7 +15224,7 @@
       <c r="I17" s="15" t="n">
         <v>61</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -15265,7 +15265,7 @@
       <c r="I18" s="20" t="n">
         <v>59</v>
       </c>
-      <c r="J18" s="24" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-27</t>
         </is>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  15 August 2026 om 07:33</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  16 August 2026 om 07:33</t>
         </is>
       </c>
     </row>
@@ -16001,9 +16001,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="D8" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="D8" s="38" t="inlineStr">
+        <is>
+          <t>1-4</t>
         </is>
       </c>
       <c r="E8" s="35" t="inlineStr">
@@ -16250,9 +16250,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="O10" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="O10" s="37" t="inlineStr">
+        <is>
+          <t>3-1</t>
         </is>
       </c>
       <c r="P10" s="35" t="inlineStr">
@@ -16725,9 +16725,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="M15" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="M15" s="38" t="inlineStr">
+        <is>
+          <t>1-2</t>
         </is>
       </c>
       <c r="N15" s="34" t="inlineStr">
@@ -17200,9 +17200,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="K20" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="K20" s="38" t="inlineStr">
+        <is>
+          <t>1-4</t>
         </is>
       </c>
       <c r="L20" s="35" t="inlineStr">
@@ -19520,7 +19520,7 @@
       <c r="I9" s="15" t="n">
         <v>48</v>
       </c>
-      <c r="J9" s="23" t="inlineStr">
+      <c r="J9" s="24" t="inlineStr">
         <is>
           <t>-7</t>
         </is>
@@ -19643,7 +19643,7 @@
       <c r="I12" s="20" t="n">
         <v>42</v>
       </c>
-      <c r="J12" s="24" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>-5</t>
         </is>
@@ -19684,7 +19684,7 @@
       <c r="I13" s="15" t="n">
         <v>49</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-1</t>
         </is>
@@ -19725,7 +19725,7 @@
       <c r="I14" s="20" t="n">
         <v>61</v>
       </c>
-      <c r="J14" s="24" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -19766,7 +19766,7 @@
       <c r="I15" s="15" t="n">
         <v>64</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -19807,7 +19807,7 @@
       <c r="I16" s="20" t="n">
         <v>55</v>
       </c>
-      <c r="J16" s="24" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-21</t>
         </is>
@@ -19848,7 +19848,7 @@
       <c r="I17" s="15" t="n">
         <v>60</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-26</t>
         </is>
@@ -19889,7 +19889,7 @@
       <c r="I18" s="20" t="n">
         <v>53</v>
       </c>
-      <c r="J18" s="24" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -22289,7 +22289,7 @@
       <c r="I10" s="20" t="n">
         <v>53</v>
       </c>
-      <c r="J10" s="24" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
@@ -22330,7 +22330,7 @@
       <c r="I11" s="15" t="n">
         <v>50</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="24" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
@@ -22412,7 +22412,7 @@
       <c r="I13" s="15" t="n">
         <v>62</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -22453,7 +22453,7 @@
       <c r="I14" s="20" t="n">
         <v>56</v>
       </c>
-      <c r="J14" s="24" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-10</t>
         </is>
@@ -22494,7 +22494,7 @@
       <c r="I15" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -22535,7 +22535,7 @@
       <c r="I16" s="20" t="n">
         <v>64</v>
       </c>
-      <c r="J16" s="24" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -22576,7 +22576,7 @@
       <c r="I17" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-16</t>
         </is>
@@ -22617,7 +22617,7 @@
       <c r="I18" s="20" t="n">
         <v>68</v>
       </c>
-      <c r="J18" s="24" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-32</t>
         </is>
@@ -25058,7 +25058,7 @@
       <c r="I11" s="15" t="n">
         <v>64</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="24" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -25099,7 +25099,7 @@
       <c r="I12" s="20" t="n">
         <v>65</v>
       </c>
-      <c r="J12" s="24" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -25140,7 +25140,7 @@
       <c r="I13" s="15" t="n">
         <v>49</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -25181,7 +25181,7 @@
       <c r="I14" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J14" s="24" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-10</t>
         </is>
@@ -25222,7 +25222,7 @@
       <c r="I15" s="15" t="n">
         <v>69</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-24</t>
         </is>
@@ -25263,7 +25263,7 @@
       <c r="I16" s="20" t="n">
         <v>59</v>
       </c>
-      <c r="J16" s="24" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -25304,7 +25304,7 @@
       <c r="I17" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-11</t>
         </is>
@@ -25345,7 +25345,7 @@
       <c r="I18" s="20" t="n">
         <v>64</v>
       </c>
-      <c r="J18" s="24" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-20</t>
         </is>
@@ -27704,7 +27704,7 @@
       <c r="I9" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J9" s="23" t="inlineStr">
+      <c r="J9" s="24" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -27745,7 +27745,7 @@
       <c r="I10" s="20" t="n">
         <v>63</v>
       </c>
-      <c r="J10" s="24" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -27786,7 +27786,7 @@
       <c r="I11" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="24" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -27868,7 +27868,7 @@
       <c r="I13" s="15" t="n">
         <v>55</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -27909,7 +27909,7 @@
       <c r="I14" s="20" t="n">
         <v>71</v>
       </c>
-      <c r="J14" s="24" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -27950,7 +27950,7 @@
       <c r="I15" s="15" t="n">
         <v>56</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-16</t>
         </is>
@@ -27991,7 +27991,7 @@
       <c r="I16" s="20" t="n">
         <v>48</v>
       </c>
-      <c r="J16" s="24" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -28032,7 +28032,7 @@
       <c r="I17" s="15" t="n">
         <v>66</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -28073,7 +28073,7 @@
       <c r="I18" s="20" t="n">
         <v>69</v>
       </c>
-      <c r="J18" s="24" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -30473,7 +30473,7 @@
       <c r="I10" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="J10" s="24" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
@@ -30514,7 +30514,7 @@
       <c r="I11" s="15" t="n">
         <v>49</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="24" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -30555,7 +30555,7 @@
       <c r="I12" s="20" t="n">
         <v>70</v>
       </c>
-      <c r="J12" s="24" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -30596,7 +30596,7 @@
       <c r="I13" s="15" t="n">
         <v>58</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
@@ -30637,7 +30637,7 @@
       <c r="I14" s="20" t="n">
         <v>62</v>
       </c>
-      <c r="J14" s="24" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-10</t>
         </is>
@@ -30678,7 +30678,7 @@
       <c r="I15" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -30719,7 +30719,7 @@
       <c r="I16" s="20" t="n">
         <v>61</v>
       </c>
-      <c r="J16" s="24" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-20</t>
         </is>
@@ -30760,7 +30760,7 @@
       <c r="I17" s="15" t="n">
         <v>67</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-29</t>
         </is>
@@ -30801,7 +30801,7 @@
       <c r="I18" s="20" t="n">
         <v>78</v>
       </c>
-      <c r="J18" s="24" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-36</t>
         </is>
@@ -31346,7 +31346,7 @@
       <c r="I11" s="15" t="n">
         <v>57</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="24" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -31387,7 +31387,7 @@
       <c r="I12" s="20" t="n">
         <v>51</v>
       </c>
-      <c r="J12" s="24" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>-8</t>
         </is>
@@ -31428,7 +31428,7 @@
       <c r="I13" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -31469,7 +31469,7 @@
       <c r="I14" s="20" t="n">
         <v>43</v>
       </c>
-      <c r="J14" s="24" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
@@ -31510,7 +31510,7 @@
       <c r="I15" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -31551,7 +31551,7 @@
       <c r="I16" s="20" t="n">
         <v>63</v>
       </c>
-      <c r="J16" s="24" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-21</t>
         </is>
@@ -31592,7 +31592,7 @@
       <c r="I17" s="15" t="n">
         <v>58</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-24</t>
         </is>
@@ -31633,7 +31633,7 @@
       <c r="I18" s="20" t="n">
         <v>56</v>
       </c>
-      <c r="J18" s="24" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -33725,21 +33725,21 @@
       </c>
       <c r="B5" s="45" t="inlineStr">
         <is>
-          <t>SBV Excelsior</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>+4</t>
+          <t>+5</t>
         </is>
       </c>
       <c r="H5" s="45" t="inlineStr">
@@ -33855,14 +33855,14 @@
       </c>
       <c r="H8" s="48" t="inlineStr">
         <is>
-          <t>SBV Excelsior</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="I8" s="18" t="n">
         <v>1</v>
       </c>
       <c r="J8" s="20" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1">
@@ -36801,7 +36801,7 @@
       <c r="I12" s="20" t="n">
         <v>56</v>
       </c>
-      <c r="J12" s="24" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -36842,7 +36842,7 @@
       <c r="I13" s="15" t="n">
         <v>70</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -36883,7 +36883,7 @@
       <c r="I14" s="20" t="n">
         <v>67</v>
       </c>
-      <c r="J14" s="24" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -36924,7 +36924,7 @@
       <c r="I15" s="15" t="n">
         <v>59</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-25</t>
         </is>
@@ -36965,7 +36965,7 @@
       <c r="I16" s="20" t="n">
         <v>75</v>
       </c>
-      <c r="J16" s="24" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-34</t>
         </is>
@@ -37006,7 +37006,7 @@
       <c r="I17" s="15" t="n">
         <v>56</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -37047,7 +37047,7 @@
       <c r="I18" s="20" t="n">
         <v>73</v>
       </c>
-      <c r="J18" s="24" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-23</t>
         </is>
@@ -39447,7 +39447,7 @@
       <c r="I10" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J10" s="24" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>-6</t>
         </is>
@@ -39488,7 +39488,7 @@
       <c r="I11" s="15" t="n">
         <v>64</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="24" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -39529,7 +39529,7 @@
       <c r="I12" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J12" s="24" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>-5</t>
         </is>
@@ -39570,7 +39570,7 @@
       <c r="I13" s="15" t="n">
         <v>56</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-10</t>
         </is>
@@ -39611,7 +39611,7 @@
       <c r="I14" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="J14" s="24" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
@@ -39652,7 +39652,7 @@
       <c r="I15" s="15" t="n">
         <v>62</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-23</t>
         </is>
@@ -39693,7 +39693,7 @@
       <c r="I16" s="20" t="n">
         <v>71</v>
       </c>
-      <c r="J16" s="24" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-29</t>
         </is>
@@ -39734,7 +39734,7 @@
       <c r="I17" s="15" t="n">
         <v>71</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-39</t>
         </is>
@@ -39775,7 +39775,7 @@
       <c r="I18" s="20" t="n">
         <v>65</v>
       </c>
-      <c r="J18" s="24" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-32</t>
         </is>
@@ -42175,7 +42175,7 @@
       <c r="I10" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J10" s="24" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -42216,7 +42216,7 @@
       <c r="I11" s="15" t="n">
         <v>70</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="24" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -42257,7 +42257,7 @@
       <c r="I12" s="20" t="n">
         <v>51</v>
       </c>
-      <c r="J12" s="24" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>-11</t>
         </is>
@@ -42298,7 +42298,7 @@
       <c r="I13" s="15" t="n">
         <v>52</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -42339,7 +42339,7 @@
       <c r="I14" s="20" t="n">
         <v>55</v>
       </c>
-      <c r="J14" s="24" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -42380,7 +42380,7 @@
       <c r="I15" s="15" t="n">
         <v>51</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -42421,7 +42421,7 @@
       <c r="I16" s="20" t="n">
         <v>48</v>
       </c>
-      <c r="J16" s="24" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -42462,7 +42462,7 @@
       <c r="I17" s="15" t="n">
         <v>67</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-31</t>
         </is>
@@ -42503,7 +42503,7 @@
       <c r="I18" s="20" t="n">
         <v>49</v>
       </c>
-      <c r="J18" s="24" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-16</t>
         </is>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 18-08-2026 07:39
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  17 August 2026 om 07:54</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  18 August 2026 om 07:39</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  17 August 2026 om 07:54</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  18 August 2026 om 07:39</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 19-08-2026 07:40
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  18 August 2026 om 07:39</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  19 August 2026 om 07:40</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  18 August 2026 om 07:39</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  19 August 2026 om 07:40</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 20-08-2026 07:43
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  19 August 2026 om 07:40</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  20 August 2026 om 07:42</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  19 August 2026 om 07:40</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  20 August 2026 om 07:42</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 21-08-2026 07:45
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  20 August 2026 om 07:42</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  21 August 2026 om 07:45</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  20 August 2026 om 07:42</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  21 August 2026 om 07:45</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 22-08-2026 07:33
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  21 August 2026 om 07:45</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  22 August 2026 om 07:33</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  21 August 2026 om 07:45</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  22 August 2026 om 07:33</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 23-08-2026 07:35
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -330,10 +330,10 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  22 August 2026 om 07:33</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  23 August 2026 om 07:35</t>
         </is>
       </c>
     </row>
@@ -990,10 +990,10 @@
         </is>
       </c>
       <c r="C3" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>0</v>
@@ -1002,17 +1002,17 @@
         <v>0</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I3" s="5" t="n">
         <v>1</v>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>+5</t>
+          <t>+7</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
@@ -1109,7 +1109,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Fortuna Sittard</t>
+          <t>AFC Ajax</t>
         </is>
       </c>
       <c r="C6" s="10" t="n">
@@ -1128,10 +1128,10 @@
         <v>4</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
@@ -1150,11 +1150,11 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>AFC Ajax</t>
+          <t>Sparta Rotterdam</t>
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D7" s="10" t="n">
         <v>1</v>
@@ -1163,25 +1163,25 @@
         <v>1</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" s="11" t="n">
         <v>4</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J7" s="12" t="inlineStr">
         <is>
-          <t>+2</t>
+          <t>+1</t>
         </is>
       </c>
       <c r="K7" s="10" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>33%</t>
         </is>
       </c>
     </row>
@@ -1269,15 +1269,15 @@
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="18" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>SC Heerenveen</t>
+          <t>Fortuna Sittard</t>
         </is>
       </c>
       <c r="C10" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D10" s="20" t="n">
         <v>1</v>
@@ -1286,25 +1286,25 @@
         <v>1</v>
       </c>
       <c r="F10" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" s="21" t="n">
         <v>4</v>
       </c>
       <c r="H10" s="20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I10" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="J10" s="22" t="inlineStr">
-        <is>
-          <t>+1</t>
+        <v>5</v>
+      </c>
+      <c r="J10" s="20" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
       <c r="K10" s="20" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>33%</t>
         </is>
       </c>
     </row>
@@ -1314,38 +1314,38 @@
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>SBV Excelsior</t>
+          <t>SC Heerenveen</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D11" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E11" s="15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" s="15" t="n">
         <v>1</v>
       </c>
       <c r="G11" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="H11" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="H11" s="15" t="n">
-        <v>5</v>
-      </c>
       <c r="I11" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="J11" s="17" t="inlineStr">
-        <is>
-          <t>+3</t>
+        <v>4</v>
+      </c>
+      <c r="J11" s="22" t="inlineStr">
+        <is>
+          <t>-1</t>
         </is>
       </c>
       <c r="K11" s="15" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>33%</t>
         </is>
       </c>
     </row>
@@ -1355,7 +1355,7 @@
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>NEC</t>
+          <t>SBV Excelsior</t>
         </is>
       </c>
       <c r="C12" s="20" t="n">
@@ -1377,11 +1377,11 @@
         <v>5</v>
       </c>
       <c r="I12" s="20" t="n">
-        <v>3</v>
-      </c>
-      <c r="J12" s="22" t="inlineStr">
-        <is>
-          <t>+2</t>
+        <v>2</v>
+      </c>
+      <c r="J12" s="23" t="inlineStr">
+        <is>
+          <t>+3</t>
         </is>
       </c>
       <c r="K12" s="20" t="inlineStr">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>FC Twente '65</t>
+          <t>NEC</t>
         </is>
       </c>
       <c r="C13" s="15" t="n">
@@ -1415,14 +1415,14 @@
         <v>3</v>
       </c>
       <c r="H13" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="I13" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I13" s="15" t="n">
-        <v>2</v>
-      </c>
       <c r="J13" s="17" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>+2</t>
         </is>
       </c>
       <c r="K13" s="15" t="inlineStr">
@@ -1433,11 +1433,11 @@
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="18" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B14" s="19" t="inlineStr">
         <is>
-          <t>Sparta Rotterdam</t>
+          <t>FC Twente '65</t>
         </is>
       </c>
       <c r="C14" s="20" t="n">
@@ -1461,7 +1461,7 @@
       <c r="I14" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="J14" s="22" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>+1</t>
         </is>
@@ -1502,7 +1502,7 @@
       <c r="I15" s="15" t="n">
         <v>4</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="22" t="inlineStr">
         <is>
           <t>-1</t>
         </is>
@@ -1519,14 +1519,14 @@
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>FC Utrecht</t>
+          <t>PEC Zwolle</t>
         </is>
       </c>
       <c r="C16" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D16" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E16" s="20" t="n">
         <v>0</v>
@@ -1535,22 +1535,22 @@
         <v>2</v>
       </c>
       <c r="G16" s="21" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H16" s="20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I16" s="20" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J16" s="24" t="inlineStr">
         <is>
-          <t>-4</t>
+          <t>-2</t>
         </is>
       </c>
       <c r="K16" s="20" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>33%</t>
         </is>
       </c>
     </row>
@@ -1560,31 +1560,31 @@
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>PEC Zwolle</t>
+          <t>FC Utrecht</t>
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D17" s="15" t="n">
         <v>0</v>
       </c>
       <c r="E17" s="15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" s="15" t="n">
         <v>2</v>
       </c>
       <c r="G17" s="16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I17" s="15" t="n">
-        <v>5</v>
-      </c>
-      <c r="J17" s="23" t="inlineStr">
+        <v>9</v>
+      </c>
+      <c r="J17" s="22" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
@@ -4025,7 +4025,7 @@
       <c r="I10" s="20" t="n">
         <v>48</v>
       </c>
-      <c r="J10" s="22" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>+1</t>
         </is>
@@ -4066,7 +4066,7 @@
       <c r="I11" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="22" t="inlineStr">
         <is>
           <t>-11</t>
         </is>
@@ -4148,7 +4148,7 @@
       <c r="I13" s="15" t="n">
         <v>58</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="22" t="inlineStr">
         <is>
           <t>-8</t>
         </is>
@@ -4230,7 +4230,7 @@
       <c r="I15" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="22" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -4312,7 +4312,7 @@
       <c r="I17" s="15" t="n">
         <v>55</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="22" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -6753,7 +6753,7 @@
       <c r="I10" s="20" t="n">
         <v>26</v>
       </c>
-      <c r="J10" s="22" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>+1</t>
         </is>
@@ -6794,7 +6794,7 @@
       <c r="I11" s="15" t="n">
         <v>41</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="22" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
@@ -6958,7 +6958,7 @@
       <c r="I15" s="15" t="n">
         <v>55</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="22" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -7040,7 +7040,7 @@
       <c r="I17" s="15" t="n">
         <v>51</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="22" t="inlineStr">
         <is>
           <t>-27</t>
         </is>
@@ -9440,7 +9440,7 @@
       <c r="I9" s="15" t="n">
         <v>68</v>
       </c>
-      <c r="J9" s="23" t="inlineStr">
+      <c r="J9" s="22" t="inlineStr">
         <is>
           <t>-7</t>
         </is>
@@ -9522,7 +9522,7 @@
       <c r="I11" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="22" t="inlineStr">
         <is>
           <t>-5</t>
         </is>
@@ -9604,7 +9604,7 @@
       <c r="I13" s="15" t="n">
         <v>73</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="22" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -9686,7 +9686,7 @@
       <c r="I15" s="15" t="n">
         <v>57</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="22" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -9768,7 +9768,7 @@
       <c r="I17" s="15" t="n">
         <v>80</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="22" t="inlineStr">
         <is>
           <t>-30</t>
         </is>
@@ -12168,7 +12168,7 @@
       <c r="I9" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J9" s="23" t="inlineStr">
+      <c r="J9" s="22" t="inlineStr">
         <is>
           <t>-8</t>
         </is>
@@ -12250,7 +12250,7 @@
       <c r="I11" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="22" t="inlineStr">
         <is>
           <t>-12</t>
         </is>
@@ -12332,7 +12332,7 @@
       <c r="I13" s="15" t="n">
         <v>56</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="22" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -12414,7 +12414,7 @@
       <c r="I15" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="22" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -12496,7 +12496,7 @@
       <c r="I17" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="22" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -14896,7 +14896,7 @@
       <c r="I9" s="15" t="n">
         <v>50</v>
       </c>
-      <c r="J9" s="23" t="inlineStr">
+      <c r="J9" s="22" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -14937,7 +14937,7 @@
       <c r="I10" s="20" t="n">
         <v>51</v>
       </c>
-      <c r="J10" s="22" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>+4</t>
         </is>
@@ -15060,7 +15060,7 @@
       <c r="I13" s="15" t="n">
         <v>59</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="22" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -15142,7 +15142,7 @@
       <c r="I15" s="15" t="n">
         <v>44</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="22" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -15224,7 +15224,7 @@
       <c r="I17" s="15" t="n">
         <v>61</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="22" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  22 August 2026 om 07:33</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  23 August 2026 om 07:35</t>
         </is>
       </c>
     </row>
@@ -16195,9 +16195,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="D10" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="D10" s="36" t="inlineStr">
+        <is>
+          <t>0-2</t>
         </is>
       </c>
       <c r="E10" s="35" t="inlineStr">
@@ -16914,9 +16914,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="L17" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="L17" s="36" t="inlineStr">
+        <is>
+          <t>0-2</t>
         </is>
       </c>
       <c r="M17" s="35" t="inlineStr">
@@ -16986,9 +16986,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="G18" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="G18" s="38" t="inlineStr">
+        <is>
+          <t>3-3</t>
         </is>
       </c>
       <c r="H18" s="36" t="inlineStr">
@@ -19520,7 +19520,7 @@
       <c r="I9" s="15" t="n">
         <v>48</v>
       </c>
-      <c r="J9" s="23" t="inlineStr">
+      <c r="J9" s="22" t="inlineStr">
         <is>
           <t>-7</t>
         </is>
@@ -19561,7 +19561,7 @@
       <c r="I10" s="20" t="n">
         <v>54</v>
       </c>
-      <c r="J10" s="22" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>+2</t>
         </is>
@@ -19684,7 +19684,7 @@
       <c r="I13" s="15" t="n">
         <v>49</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="22" t="inlineStr">
         <is>
           <t>-1</t>
         </is>
@@ -19766,7 +19766,7 @@
       <c r="I15" s="15" t="n">
         <v>64</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="22" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -19848,7 +19848,7 @@
       <c r="I17" s="15" t="n">
         <v>60</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="22" t="inlineStr">
         <is>
           <t>-26</t>
         </is>
@@ -22330,7 +22330,7 @@
       <c r="I11" s="15" t="n">
         <v>50</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="22" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
@@ -22371,7 +22371,7 @@
       <c r="I12" s="20" t="n">
         <v>51</v>
       </c>
-      <c r="J12" s="22" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>+5</t>
         </is>
@@ -22412,7 +22412,7 @@
       <c r="I13" s="15" t="n">
         <v>62</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="22" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -22494,7 +22494,7 @@
       <c r="I15" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="22" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -22576,7 +22576,7 @@
       <c r="I17" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="22" t="inlineStr">
         <is>
           <t>-16</t>
         </is>
@@ -25017,7 +25017,7 @@
       <c r="I10" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J10" s="22" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>+4</t>
         </is>
@@ -25058,7 +25058,7 @@
       <c r="I11" s="15" t="n">
         <v>64</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="22" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -25140,7 +25140,7 @@
       <c r="I13" s="15" t="n">
         <v>49</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="22" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -25222,7 +25222,7 @@
       <c r="I15" s="15" t="n">
         <v>69</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="22" t="inlineStr">
         <is>
           <t>-24</t>
         </is>
@@ -25304,7 +25304,7 @@
       <c r="I17" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="22" t="inlineStr">
         <is>
           <t>-11</t>
         </is>
@@ -27704,7 +27704,7 @@
       <c r="I9" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J9" s="23" t="inlineStr">
+      <c r="J9" s="22" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -27786,7 +27786,7 @@
       <c r="I11" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="22" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -27827,7 +27827,7 @@
       <c r="I12" s="20" t="n">
         <v>54</v>
       </c>
-      <c r="J12" s="22" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>+2</t>
         </is>
@@ -27868,7 +27868,7 @@
       <c r="I13" s="15" t="n">
         <v>55</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="22" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -27950,7 +27950,7 @@
       <c r="I15" s="15" t="n">
         <v>56</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="22" t="inlineStr">
         <is>
           <t>-16</t>
         </is>
@@ -28032,7 +28032,7 @@
       <c r="I17" s="15" t="n">
         <v>66</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="22" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -30514,7 +30514,7 @@
       <c r="I11" s="15" t="n">
         <v>49</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="22" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -30596,7 +30596,7 @@
       <c r="I13" s="15" t="n">
         <v>58</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="22" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
@@ -30678,7 +30678,7 @@
       <c r="I15" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="22" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -30760,7 +30760,7 @@
       <c r="I17" s="15" t="n">
         <v>67</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="22" t="inlineStr">
         <is>
           <t>-29</t>
         </is>
@@ -31305,7 +31305,7 @@
       <c r="I10" s="20" t="n">
         <v>46</v>
       </c>
-      <c r="J10" s="22" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>+5</t>
         </is>
@@ -31346,7 +31346,7 @@
       <c r="I11" s="15" t="n">
         <v>57</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="22" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -31428,7 +31428,7 @@
       <c r="I13" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="22" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -31510,7 +31510,7 @@
       <c r="I15" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="22" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -31592,7 +31592,7 @@
       <c r="I17" s="15" t="n">
         <v>58</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="22" t="inlineStr">
         <is>
           <t>-24</t>
         </is>
@@ -33729,17 +33729,17 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E5" s="5" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>+5</t>
+          <t>+7</t>
         </is>
       </c>
       <c r="H5" s="45" t="inlineStr">
@@ -36719,7 +36719,7 @@
       <c r="I10" s="20" t="n">
         <v>48</v>
       </c>
-      <c r="J10" s="22" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>+3</t>
         </is>
@@ -36842,7 +36842,7 @@
       <c r="I13" s="15" t="n">
         <v>70</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="22" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -36924,7 +36924,7 @@
       <c r="I15" s="15" t="n">
         <v>59</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="22" t="inlineStr">
         <is>
           <t>-25</t>
         </is>
@@ -37006,7 +37006,7 @@
       <c r="I17" s="15" t="n">
         <v>56</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="22" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -39488,7 +39488,7 @@
       <c r="I11" s="15" t="n">
         <v>64</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="22" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -39570,7 +39570,7 @@
       <c r="I13" s="15" t="n">
         <v>56</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="22" t="inlineStr">
         <is>
           <t>-10</t>
         </is>
@@ -39652,7 +39652,7 @@
       <c r="I15" s="15" t="n">
         <v>62</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="22" t="inlineStr">
         <is>
           <t>-23</t>
         </is>
@@ -39734,7 +39734,7 @@
       <c r="I17" s="15" t="n">
         <v>71</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="22" t="inlineStr">
         <is>
           <t>-39</t>
         </is>
@@ -42216,7 +42216,7 @@
       <c r="I11" s="15" t="n">
         <v>70</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="22" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -42298,7 +42298,7 @@
       <c r="I13" s="15" t="n">
         <v>52</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="22" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -42380,7 +42380,7 @@
       <c r="I15" s="15" t="n">
         <v>51</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="22" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -42462,7 +42462,7 @@
       <c r="I17" s="15" t="n">
         <v>67</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="22" t="inlineStr">
         <is>
           <t>-31</t>
         </is>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 24-08-2026 07:58
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  23 August 2026 om 07:35</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  24 August 2026 om 07:58</t>
         </is>
       </c>
     </row>
@@ -1027,55 +1027,55 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>FC Groningen</t>
+          <t>Go Ahead Eagles</t>
         </is>
       </c>
       <c r="C4" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D4" s="10" t="n">
         <v>2</v>
       </c>
       <c r="E4" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" s="10" t="n">
         <v>0</v>
       </c>
       <c r="G4" s="11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="I4" s="10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J4" s="12" t="inlineStr">
         <is>
-          <t>+4</t>
+          <t>+5</t>
         </is>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>67%</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>PSV</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Go Ahead Eagles</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="n">
+      <c r="D5" s="10" t="n">
         <v>2</v>
-      </c>
-      <c r="D5" s="10" t="n">
-        <v>1</v>
       </c>
       <c r="E5" s="10" t="n">
         <v>1</v>
@@ -1084,22 +1084,22 @@
         <v>0</v>
       </c>
       <c r="G5" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="H5" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="I5" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="H5" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="I5" s="10" t="n">
-        <v>3</v>
-      </c>
       <c r="J5" s="12" t="inlineStr">
         <is>
-          <t>+3</t>
+          <t>+5</t>
         </is>
       </c>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>67%</t>
         </is>
       </c>
     </row>
@@ -1109,14 +1109,14 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>AFC Ajax</t>
+          <t>Feyenoord Rotterdam</t>
         </is>
       </c>
       <c r="C6" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" s="10" t="n">
         <v>2</v>
-      </c>
-      <c r="D6" s="10" t="n">
-        <v>1</v>
       </c>
       <c r="E6" s="10" t="n">
         <v>1</v>
@@ -1125,22 +1125,22 @@
         <v>0</v>
       </c>
       <c r="G6" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="H6" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="I6" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="H6" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="I6" s="10" t="n">
-        <v>2</v>
-      </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
-          <t>+2</t>
+          <t>+4</t>
         </is>
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>67%</t>
         </is>
       </c>
     </row>
@@ -1150,38 +1150,38 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Sparta Rotterdam</t>
+          <t>FC Groningen</t>
         </is>
       </c>
       <c r="C7" s="10" t="n">
         <v>3</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" s="10" t="n">
         <v>1</v>
       </c>
       <c r="G7" s="11" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>5</v>
-      </c>
-      <c r="J7" s="12" t="inlineStr">
-        <is>
-          <t>+1</t>
+        <v>7</v>
+      </c>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
       <c r="K7" s="10" t="inlineStr">
         <is>
-          <t>33%</t>
+          <t>67%</t>
         </is>
       </c>
     </row>
@@ -1191,7 +1191,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>PSV</t>
+          <t>AFC Ajax</t>
         </is>
       </c>
       <c r="C8" s="10" t="n">
@@ -1213,11 +1213,11 @@
         <v>4</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J8" s="12" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>+2</t>
         </is>
       </c>
       <c r="K8" s="10" t="inlineStr">
@@ -1232,11 +1232,11 @@
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>Feyenoord Rotterdam</t>
+          <t>Sparta Rotterdam</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D9" s="15" t="n">
         <v>1</v>
@@ -1245,16 +1245,16 @@
         <v>1</v>
       </c>
       <c r="F9" s="15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" s="16" t="n">
         <v>4</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I9" s="15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J9" s="17" t="inlineStr">
         <is>
@@ -1263,7 +1263,7 @@
       </c>
       <c r="K9" s="15" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>33%</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>ADO Den Haag</t>
+          <t>Willem II Tilburg</t>
         </is>
       </c>
       <c r="C18" s="20" t="n">
@@ -1620,14 +1620,14 @@
         <v>0</v>
       </c>
       <c r="H18" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I18" s="20" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J18" s="24" t="inlineStr">
         <is>
-          <t>-5</t>
+          <t>-6</t>
         </is>
       </c>
       <c r="K18" s="20" t="inlineStr">
@@ -1642,11 +1642,11 @@
       </c>
       <c r="B19" s="26" t="inlineStr">
         <is>
-          <t>Willem II Tilburg</t>
+          <t>ADO Den Haag</t>
         </is>
       </c>
       <c r="C19" s="27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D19" s="27" t="n">
         <v>0</v>
@@ -1655,7 +1655,7 @@
         <v>0</v>
       </c>
       <c r="F19" s="27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G19" s="28" t="n">
         <v>0</v>
@@ -1664,11 +1664,11 @@
         <v>2</v>
       </c>
       <c r="I19" s="27" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J19" s="29" t="inlineStr">
         <is>
-          <t>-6</t>
+          <t>-7</t>
         </is>
       </c>
       <c r="K19" s="27" t="inlineStr">
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="C20" s="27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D20" s="27" t="n">
         <v>0</v>
@@ -1696,20 +1696,20 @@
         <v>0</v>
       </c>
       <c r="F20" s="27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G20" s="28" t="n">
         <v>0</v>
       </c>
       <c r="H20" s="27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I20" s="27" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="J20" s="29" t="inlineStr">
         <is>
-          <t>-6</t>
+          <t>-9</t>
         </is>
       </c>
       <c r="K20" s="27" t="inlineStr">
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  23 August 2026 om 07:35</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  24 August 2026 om 07:58</t>
         </is>
       </c>
     </row>
@@ -16282,9 +16282,9 @@
           <t>Go Ahead Eagles</t>
         </is>
       </c>
-      <c r="B11" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="B11" s="39" t="inlineStr">
+        <is>
+          <t>3-1</t>
         </is>
       </c>
       <c r="C11" s="35" t="inlineStr">
@@ -16588,9 +16588,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="E14" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="E14" s="39" t="inlineStr">
+        <is>
+          <t>5-1</t>
         </is>
       </c>
       <c r="F14" s="35" t="inlineStr">
@@ -16797,9 +16797,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="H16" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="H16" s="36" t="inlineStr">
+        <is>
+          <t>2-5</t>
         </is>
       </c>
       <c r="I16" s="35" t="inlineStr">

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 25-08-2026 07:46
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  24 August 2026 om 07:58</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  25 August 2026 om 07:46</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  24 August 2026 om 07:58</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  25 August 2026 om 07:46</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 26-08-2026 07:49
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  25 August 2026 om 07:46</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  26 August 2026 om 07:49</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  25 August 2026 om 07:46</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  26 August 2026 om 07:49</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 27-08-2026 18:09
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  26 August 2026 om 07:49</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  27 August 2026 om 18:09</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  26 August 2026 om 07:49</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  27 August 2026 om 18:09</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 29-08-2026 13:02
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  28 August 2026 om 19:19</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  29 August 2026 om 13:02</t>
         </is>
       </c>
     </row>
@@ -1169,10 +1169,10 @@
         <v>7</v>
       </c>
       <c r="H7" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="I7" s="10" t="n">
         <v>7</v>
-      </c>
-      <c r="I7" s="10" t="n">
-        <v>6</v>
       </c>
       <c r="J7" s="12" t="inlineStr">
         <is>
@@ -1210,10 +1210,10 @@
         <v>6</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J8" s="13" t="inlineStr">
         <is>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="31" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  28 August 2026 om 19:19</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  29 August 2026 om 13:02</t>
         </is>
       </c>
     </row>
@@ -15832,9 +15832,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="I6" s="36" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="I6" s="37" t="inlineStr">
+        <is>
+          <t>2-3</t>
         </is>
       </c>
       <c r="J6" s="36" t="inlineStr">

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 31-08-2026 14:55
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -330,13 +330,13 @@
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  30 August 2026 om 12:39</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  31 August 2026 om 14:55</t>
         </is>
       </c>
     </row>
@@ -1087,10 +1087,10 @@
         <v>8</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J5" s="12" t="inlineStr">
         <is>
@@ -1109,11 +1109,11 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Go Ahead Eagles</t>
+          <t>AFC Ajax</t>
         </is>
       </c>
       <c r="C6" s="10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D6" s="10" t="n">
         <v>2</v>
@@ -1122,25 +1122,25 @@
         <v>1</v>
       </c>
       <c r="F6" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" s="11" t="n">
         <v>7</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
-          <t>+2</t>
+          <t>+6</t>
         </is>
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>67%</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Fortuna Sittard</t>
+          <t>Go Ahead Eagles</t>
         </is>
       </c>
       <c r="C7" s="10" t="n">
@@ -1169,14 +1169,14 @@
         <v>7</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="J7" s="12" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>+2</t>
         </is>
       </c>
       <c r="K7" s="10" t="inlineStr">
@@ -1191,38 +1191,38 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>NEC</t>
+          <t>Fortuna Sittard</t>
         </is>
       </c>
       <c r="C8" s="10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D8" s="10" t="n">
         <v>2</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" s="10" t="n">
         <v>1</v>
       </c>
       <c r="G8" s="11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H8" s="10" t="n">
         <v>8</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J8" s="12" t="inlineStr">
         <is>
-          <t>+4</t>
+          <t>+1</t>
         </is>
       </c>
       <c r="K8" s="10" t="inlineStr">
         <is>
-          <t>67%</t>
+          <t>50%</t>
         </is>
       </c>
     </row>
@@ -1232,7 +1232,7 @@
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>SBV Excelsior</t>
+          <t>NEC</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
@@ -1251,10 +1251,10 @@
         <v>6</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I9" s="15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J9" s="17" t="inlineStr">
         <is>
@@ -1273,11 +1273,11 @@
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>FC Groningen</t>
+          <t>FC Twente '65</t>
         </is>
       </c>
       <c r="C10" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D10" s="20" t="n">
         <v>2</v>
@@ -1286,66 +1286,66 @@
         <v>0</v>
       </c>
       <c r="F10" s="20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G10" s="21" t="n">
         <v>6</v>
       </c>
       <c r="H10" s="20" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I10" s="20" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="J10" s="22" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>+4</t>
         </is>
       </c>
       <c r="K10" s="20" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>67%</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="13" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>SC Heerenveen</t>
+          <t>SBV Excelsior</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D11" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E11" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F11" s="15" t="n">
         <v>1</v>
       </c>
       <c r="G11" s="16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H11" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="I11" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="I11" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="J11" s="23" t="inlineStr">
-        <is>
-          <t>-1</t>
+      <c r="J11" s="17" t="inlineStr">
+        <is>
+          <t>+4</t>
         </is>
       </c>
       <c r="K11" s="15" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>67%</t>
         </is>
       </c>
     </row>
@@ -1355,33 +1355,33 @@
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>AFC Ajax</t>
+          <t>FC Groningen</t>
         </is>
       </c>
       <c r="C12" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="20" t="n">
-        <v>1</v>
-      </c>
       <c r="E12" s="20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12" s="20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G12" s="21" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H12" s="20" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="I12" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="J12" s="24" t="inlineStr">
-        <is>
-          <t>+2</t>
+        <v>10</v>
+      </c>
+      <c r="J12" s="23" t="inlineStr">
+        <is>
+          <t>-1</t>
         </is>
       </c>
       <c r="K12" s="20" t="inlineStr">
@@ -1396,7 +1396,7 @@
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>Sparta Rotterdam</t>
+          <t>SC Heerenveen</t>
         </is>
       </c>
       <c r="C13" s="15" t="n">
@@ -1406,23 +1406,23 @@
         <v>1</v>
       </c>
       <c r="E13" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F13" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="F13" s="15" t="n">
-        <v>2</v>
-      </c>
       <c r="G13" s="16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I13" s="15" t="n">
-        <v>7</v>
-      </c>
-      <c r="J13" s="15" t="inlineStr">
-        <is>
-          <t>0</t>
+        <v>6</v>
+      </c>
+      <c r="J13" s="24" t="inlineStr">
+        <is>
+          <t>-1</t>
         </is>
       </c>
       <c r="K13" s="15" t="inlineStr">
@@ -1437,38 +1437,38 @@
       </c>
       <c r="B14" s="19" t="inlineStr">
         <is>
-          <t>FC Twente '65</t>
+          <t>Sparta Rotterdam</t>
         </is>
       </c>
       <c r="C14" s="20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D14" s="20" t="n">
         <v>1</v>
       </c>
       <c r="E14" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" s="20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G14" s="21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H14" s="20" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="I14" s="20" t="n">
-        <v>2</v>
-      </c>
-      <c r="J14" s="24" t="inlineStr">
-        <is>
-          <t>+1</t>
+        <v>7</v>
+      </c>
+      <c r="J14" s="20" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
       <c r="K14" s="20" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>25%</t>
         </is>
       </c>
     </row>
@@ -1478,11 +1478,11 @@
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>Telstar 1963</t>
+          <t>PEC Zwolle</t>
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D15" s="15" t="n">
         <v>1</v>
@@ -1491,25 +1491,25 @@
         <v>0</v>
       </c>
       <c r="F15" s="15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G15" s="16" t="n">
         <v>3</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I15" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="J15" s="23" t="inlineStr">
-        <is>
-          <t>-1</t>
+        <v>8</v>
+      </c>
+      <c r="J15" s="24" t="inlineStr">
+        <is>
+          <t>-4</t>
         </is>
       </c>
       <c r="K15" s="15" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>25%</t>
         </is>
       </c>
     </row>
@@ -1519,11 +1519,11 @@
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>PEC Zwolle</t>
+          <t>Telstar 1963</t>
         </is>
       </c>
       <c r="C16" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D16" s="20" t="n">
         <v>1</v>
@@ -1532,25 +1532,25 @@
         <v>0</v>
       </c>
       <c r="F16" s="20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G16" s="21" t="n">
         <v>3</v>
       </c>
       <c r="H16" s="20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I16" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="J16" s="22" t="inlineStr">
-        <is>
-          <t>-4</t>
+      <c r="J16" s="23" t="inlineStr">
+        <is>
+          <t>-5</t>
         </is>
       </c>
       <c r="K16" s="20" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>33%</t>
         </is>
       </c>
     </row>
@@ -1579,12 +1579,12 @@
         <v>1</v>
       </c>
       <c r="H17" s="15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I17" s="15" t="n">
-        <v>8</v>
-      </c>
-      <c r="J17" s="23" t="inlineStr">
+        <v>10</v>
+      </c>
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-6</t>
         </is>
@@ -1620,12 +1620,12 @@
         <v>1</v>
       </c>
       <c r="H18" s="20" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I18" s="20" t="n">
-        <v>9</v>
-      </c>
-      <c r="J18" s="22" t="inlineStr">
+        <v>11</v>
+      </c>
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-7</t>
         </is>
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="C20" s="27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D20" s="27" t="n">
         <v>0</v>
@@ -1696,20 +1696,20 @@
         <v>0</v>
       </c>
       <c r="F20" s="27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G20" s="28" t="n">
         <v>0</v>
       </c>
       <c r="H20" s="27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I20" s="27" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="J20" s="29" t="inlineStr">
         <is>
-          <t>-9</t>
+          <t>-12</t>
         </is>
       </c>
       <c r="K20" s="27" t="inlineStr">
@@ -4025,7 +4025,7 @@
       <c r="I10" s="20" t="n">
         <v>48</v>
       </c>
-      <c r="J10" s="24" t="inlineStr">
+      <c r="J10" s="22" t="inlineStr">
         <is>
           <t>+1</t>
         </is>
@@ -4066,7 +4066,7 @@
       <c r="I11" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="24" t="inlineStr">
         <is>
           <t>-11</t>
         </is>
@@ -4107,7 +4107,7 @@
       <c r="I12" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J12" s="22" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -4148,7 +4148,7 @@
       <c r="I13" s="15" t="n">
         <v>58</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-8</t>
         </is>
@@ -4189,7 +4189,7 @@
       <c r="I14" s="20" t="n">
         <v>49</v>
       </c>
-      <c r="J14" s="22" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-6</t>
         </is>
@@ -4230,7 +4230,7 @@
       <c r="I15" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -4271,7 +4271,7 @@
       <c r="I16" s="20" t="n">
         <v>68</v>
       </c>
-      <c r="J16" s="22" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-28</t>
         </is>
@@ -4312,7 +4312,7 @@
       <c r="I17" s="15" t="n">
         <v>55</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -4353,7 +4353,7 @@
       <c r="I18" s="20" t="n">
         <v>68</v>
       </c>
-      <c r="J18" s="22" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-28</t>
         </is>
@@ -6753,7 +6753,7 @@
       <c r="I10" s="20" t="n">
         <v>26</v>
       </c>
-      <c r="J10" s="24" t="inlineStr">
+      <c r="J10" s="22" t="inlineStr">
         <is>
           <t>+1</t>
         </is>
@@ -6794,7 +6794,7 @@
       <c r="I11" s="15" t="n">
         <v>41</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="24" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
@@ -6835,7 +6835,7 @@
       <c r="I12" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="J12" s="22" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
@@ -6917,7 +6917,7 @@
       <c r="I14" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="J14" s="22" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -6958,7 +6958,7 @@
       <c r="I15" s="15" t="n">
         <v>55</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -6999,7 +6999,7 @@
       <c r="I16" s="20" t="n">
         <v>52</v>
       </c>
-      <c r="J16" s="22" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-23</t>
         </is>
@@ -7040,7 +7040,7 @@
       <c r="I17" s="15" t="n">
         <v>51</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-27</t>
         </is>
@@ -7081,7 +7081,7 @@
       <c r="I18" s="20" t="n">
         <v>46</v>
       </c>
-      <c r="J18" s="22" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-12</t>
         </is>
@@ -9440,7 +9440,7 @@
       <c r="I9" s="15" t="n">
         <v>68</v>
       </c>
-      <c r="J9" s="23" t="inlineStr">
+      <c r="J9" s="24" t="inlineStr">
         <is>
           <t>-7</t>
         </is>
@@ -9481,7 +9481,7 @@
       <c r="I10" s="20" t="n">
         <v>41</v>
       </c>
-      <c r="J10" s="22" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -9522,7 +9522,7 @@
       <c r="I11" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="24" t="inlineStr">
         <is>
           <t>-5</t>
         </is>
@@ -9563,7 +9563,7 @@
       <c r="I12" s="20" t="n">
         <v>72</v>
       </c>
-      <c r="J12" s="22" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -9604,7 +9604,7 @@
       <c r="I13" s="15" t="n">
         <v>73</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -9645,7 +9645,7 @@
       <c r="I14" s="20" t="n">
         <v>63</v>
       </c>
-      <c r="J14" s="22" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-16</t>
         </is>
@@ -9686,7 +9686,7 @@
       <c r="I15" s="15" t="n">
         <v>57</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -9727,7 +9727,7 @@
       <c r="I16" s="20" t="n">
         <v>72</v>
       </c>
-      <c r="J16" s="22" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-31</t>
         </is>
@@ -9768,7 +9768,7 @@
       <c r="I17" s="15" t="n">
         <v>80</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-30</t>
         </is>
@@ -9809,7 +9809,7 @@
       <c r="I18" s="20" t="n">
         <v>79</v>
       </c>
-      <c r="J18" s="22" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-33</t>
         </is>
@@ -12168,7 +12168,7 @@
       <c r="I9" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J9" s="23" t="inlineStr">
+      <c r="J9" s="24" t="inlineStr">
         <is>
           <t>-8</t>
         </is>
@@ -12209,7 +12209,7 @@
       <c r="I10" s="20" t="n">
         <v>53</v>
       </c>
-      <c r="J10" s="22" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>-5</t>
         </is>
@@ -12250,7 +12250,7 @@
       <c r="I11" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="24" t="inlineStr">
         <is>
           <t>-12</t>
         </is>
@@ -12291,7 +12291,7 @@
       <c r="I12" s="20" t="n">
         <v>64</v>
       </c>
-      <c r="J12" s="22" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -12332,7 +12332,7 @@
       <c r="I13" s="15" t="n">
         <v>56</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -12414,7 +12414,7 @@
       <c r="I15" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -12455,7 +12455,7 @@
       <c r="I16" s="20" t="n">
         <v>57</v>
       </c>
-      <c r="J16" s="22" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-16</t>
         </is>
@@ -12496,7 +12496,7 @@
       <c r="I17" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -12537,7 +12537,7 @@
       <c r="I18" s="20" t="n">
         <v>69</v>
       </c>
-      <c r="J18" s="22" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-27</t>
         </is>
@@ -14896,7 +14896,7 @@
       <c r="I9" s="15" t="n">
         <v>50</v>
       </c>
-      <c r="J9" s="23" t="inlineStr">
+      <c r="J9" s="24" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -14937,7 +14937,7 @@
       <c r="I10" s="20" t="n">
         <v>51</v>
       </c>
-      <c r="J10" s="24" t="inlineStr">
+      <c r="J10" s="22" t="inlineStr">
         <is>
           <t>+4</t>
         </is>
@@ -15019,7 +15019,7 @@
       <c r="I12" s="20" t="n">
         <v>55</v>
       </c>
-      <c r="J12" s="22" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -15060,7 +15060,7 @@
       <c r="I13" s="15" t="n">
         <v>59</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -15101,7 +15101,7 @@
       <c r="I14" s="20" t="n">
         <v>60</v>
       </c>
-      <c r="J14" s="22" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -15142,7 +15142,7 @@
       <c r="I15" s="15" t="n">
         <v>44</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -15183,7 +15183,7 @@
       <c r="I16" s="20" t="n">
         <v>67</v>
       </c>
-      <c r="J16" s="22" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-28</t>
         </is>
@@ -15224,7 +15224,7 @@
       <c r="I17" s="15" t="n">
         <v>61</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -15265,7 +15265,7 @@
       <c r="I18" s="20" t="n">
         <v>59</v>
       </c>
-      <c r="J18" s="22" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-27</t>
         </is>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  30 August 2026 om 12:39</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  31 August 2026 om 14:55</t>
         </is>
       </c>
     </row>
@@ -15740,9 +15740,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="J5" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="J5" s="39" t="inlineStr">
+        <is>
+          <t>5-2</t>
         </is>
       </c>
       <c r="K5" s="35" t="inlineStr">
@@ -15832,9 +15832,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="I6" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="I6" s="36" t="inlineStr">
+        <is>
+          <t>2-3</t>
         </is>
       </c>
       <c r="J6" s="35" t="inlineStr">
@@ -16088,9 +16088,9 @@
           <t>Feyenoord Rotterdam</t>
         </is>
       </c>
-      <c r="B9" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="B9" s="38" t="inlineStr">
+        <is>
+          <t>2-2</t>
         </is>
       </c>
       <c r="C9" s="35" t="inlineStr">
@@ -16521,9 +16521,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="K13" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="K13" s="36" t="inlineStr">
+        <is>
+          <t>1-3</t>
         </is>
       </c>
       <c r="L13" s="34" t="inlineStr">
@@ -16745,9 +16745,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="Q15" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="Q15" s="39" t="inlineStr">
+        <is>
+          <t>2-1</t>
         </is>
       </c>
       <c r="R15" s="35" t="inlineStr">
@@ -17063,9 +17063,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="C19" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="C19" s="36" t="inlineStr">
+        <is>
+          <t>0-4</t>
         </is>
       </c>
       <c r="D19" s="35" t="inlineStr">
@@ -17225,9 +17225,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="P20" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="P20" s="38" t="inlineStr">
+        <is>
+          <t>2-2</t>
         </is>
       </c>
       <c r="Q20" s="35" t="inlineStr">
@@ -19520,7 +19520,7 @@
       <c r="I9" s="15" t="n">
         <v>48</v>
       </c>
-      <c r="J9" s="23" t="inlineStr">
+      <c r="J9" s="24" t="inlineStr">
         <is>
           <t>-7</t>
         </is>
@@ -19561,7 +19561,7 @@
       <c r="I10" s="20" t="n">
         <v>54</v>
       </c>
-      <c r="J10" s="24" t="inlineStr">
+      <c r="J10" s="22" t="inlineStr">
         <is>
           <t>+2</t>
         </is>
@@ -19643,7 +19643,7 @@
       <c r="I12" s="20" t="n">
         <v>42</v>
       </c>
-      <c r="J12" s="22" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>-5</t>
         </is>
@@ -19684,7 +19684,7 @@
       <c r="I13" s="15" t="n">
         <v>49</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-1</t>
         </is>
@@ -19725,7 +19725,7 @@
       <c r="I14" s="20" t="n">
         <v>61</v>
       </c>
-      <c r="J14" s="22" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -19766,7 +19766,7 @@
       <c r="I15" s="15" t="n">
         <v>64</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -19807,7 +19807,7 @@
       <c r="I16" s="20" t="n">
         <v>55</v>
       </c>
-      <c r="J16" s="22" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-21</t>
         </is>
@@ -19848,7 +19848,7 @@
       <c r="I17" s="15" t="n">
         <v>60</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-26</t>
         </is>
@@ -19889,7 +19889,7 @@
       <c r="I18" s="20" t="n">
         <v>53</v>
       </c>
-      <c r="J18" s="22" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -22289,7 +22289,7 @@
       <c r="I10" s="20" t="n">
         <v>53</v>
       </c>
-      <c r="J10" s="22" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
@@ -22330,7 +22330,7 @@
       <c r="I11" s="15" t="n">
         <v>50</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="24" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
@@ -22371,7 +22371,7 @@
       <c r="I12" s="20" t="n">
         <v>51</v>
       </c>
-      <c r="J12" s="24" t="inlineStr">
+      <c r="J12" s="22" t="inlineStr">
         <is>
           <t>+5</t>
         </is>
@@ -22412,7 +22412,7 @@
       <c r="I13" s="15" t="n">
         <v>62</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -22453,7 +22453,7 @@
       <c r="I14" s="20" t="n">
         <v>56</v>
       </c>
-      <c r="J14" s="22" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-10</t>
         </is>
@@ -22494,7 +22494,7 @@
       <c r="I15" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -22535,7 +22535,7 @@
       <c r="I16" s="20" t="n">
         <v>64</v>
       </c>
-      <c r="J16" s="22" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -22576,7 +22576,7 @@
       <c r="I17" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-16</t>
         </is>
@@ -22617,7 +22617,7 @@
       <c r="I18" s="20" t="n">
         <v>68</v>
       </c>
-      <c r="J18" s="22" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-32</t>
         </is>
@@ -25017,7 +25017,7 @@
       <c r="I10" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J10" s="24" t="inlineStr">
+      <c r="J10" s="22" t="inlineStr">
         <is>
           <t>+4</t>
         </is>
@@ -25058,7 +25058,7 @@
       <c r="I11" s="15" t="n">
         <v>64</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="24" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -25099,7 +25099,7 @@
       <c r="I12" s="20" t="n">
         <v>65</v>
       </c>
-      <c r="J12" s="22" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -25140,7 +25140,7 @@
       <c r="I13" s="15" t="n">
         <v>49</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -25181,7 +25181,7 @@
       <c r="I14" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J14" s="22" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-10</t>
         </is>
@@ -25222,7 +25222,7 @@
       <c r="I15" s="15" t="n">
         <v>69</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-24</t>
         </is>
@@ -25263,7 +25263,7 @@
       <c r="I16" s="20" t="n">
         <v>59</v>
       </c>
-      <c r="J16" s="22" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -25304,7 +25304,7 @@
       <c r="I17" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-11</t>
         </is>
@@ -25345,7 +25345,7 @@
       <c r="I18" s="20" t="n">
         <v>64</v>
       </c>
-      <c r="J18" s="22" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-20</t>
         </is>
@@ -27704,7 +27704,7 @@
       <c r="I9" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J9" s="23" t="inlineStr">
+      <c r="J9" s="24" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -27745,7 +27745,7 @@
       <c r="I10" s="20" t="n">
         <v>63</v>
       </c>
-      <c r="J10" s="22" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -27786,7 +27786,7 @@
       <c r="I11" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="24" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -27827,7 +27827,7 @@
       <c r="I12" s="20" t="n">
         <v>54</v>
       </c>
-      <c r="J12" s="24" t="inlineStr">
+      <c r="J12" s="22" t="inlineStr">
         <is>
           <t>+2</t>
         </is>
@@ -27868,7 +27868,7 @@
       <c r="I13" s="15" t="n">
         <v>55</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -27909,7 +27909,7 @@
       <c r="I14" s="20" t="n">
         <v>71</v>
       </c>
-      <c r="J14" s="22" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -27950,7 +27950,7 @@
       <c r="I15" s="15" t="n">
         <v>56</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-16</t>
         </is>
@@ -27991,7 +27991,7 @@
       <c r="I16" s="20" t="n">
         <v>48</v>
       </c>
-      <c r="J16" s="22" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -28032,7 +28032,7 @@
       <c r="I17" s="15" t="n">
         <v>66</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -28073,7 +28073,7 @@
       <c r="I18" s="20" t="n">
         <v>69</v>
       </c>
-      <c r="J18" s="22" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -30473,7 +30473,7 @@
       <c r="I10" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="J10" s="22" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
@@ -30514,7 +30514,7 @@
       <c r="I11" s="15" t="n">
         <v>49</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="24" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -30555,7 +30555,7 @@
       <c r="I12" s="20" t="n">
         <v>70</v>
       </c>
-      <c r="J12" s="22" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -30596,7 +30596,7 @@
       <c r="I13" s="15" t="n">
         <v>58</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
@@ -30637,7 +30637,7 @@
       <c r="I14" s="20" t="n">
         <v>62</v>
       </c>
-      <c r="J14" s="22" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-10</t>
         </is>
@@ -30678,7 +30678,7 @@
       <c r="I15" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -30719,7 +30719,7 @@
       <c r="I16" s="20" t="n">
         <v>61</v>
       </c>
-      <c r="J16" s="22" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-20</t>
         </is>
@@ -30760,7 +30760,7 @@
       <c r="I17" s="15" t="n">
         <v>67</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-29</t>
         </is>
@@ -30801,7 +30801,7 @@
       <c r="I18" s="20" t="n">
         <v>78</v>
       </c>
-      <c r="J18" s="22" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-36</t>
         </is>
@@ -31305,7 +31305,7 @@
       <c r="I10" s="20" t="n">
         <v>46</v>
       </c>
-      <c r="J10" s="24" t="inlineStr">
+      <c r="J10" s="22" t="inlineStr">
         <is>
           <t>+5</t>
         </is>
@@ -31346,7 +31346,7 @@
       <c r="I11" s="15" t="n">
         <v>57</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="24" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -31387,7 +31387,7 @@
       <c r="I12" s="20" t="n">
         <v>51</v>
       </c>
-      <c r="J12" s="22" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>-8</t>
         </is>
@@ -31428,7 +31428,7 @@
       <c r="I13" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -31469,7 +31469,7 @@
       <c r="I14" s="20" t="n">
         <v>43</v>
       </c>
-      <c r="J14" s="22" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
@@ -31510,7 +31510,7 @@
       <c r="I15" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -31551,7 +31551,7 @@
       <c r="I16" s="20" t="n">
         <v>63</v>
       </c>
-      <c r="J16" s="22" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-21</t>
         </is>
@@ -31592,7 +31592,7 @@
       <c r="I17" s="15" t="n">
         <v>58</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-24</t>
         </is>
@@ -31633,7 +31633,7 @@
       <c r="I18" s="20" t="n">
         <v>56</v>
       </c>
-      <c r="J18" s="22" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -36719,7 +36719,7 @@
       <c r="I10" s="20" t="n">
         <v>48</v>
       </c>
-      <c r="J10" s="24" t="inlineStr">
+      <c r="J10" s="22" t="inlineStr">
         <is>
           <t>+3</t>
         </is>
@@ -36801,7 +36801,7 @@
       <c r="I12" s="20" t="n">
         <v>56</v>
       </c>
-      <c r="J12" s="22" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -36842,7 +36842,7 @@
       <c r="I13" s="15" t="n">
         <v>70</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -36883,7 +36883,7 @@
       <c r="I14" s="20" t="n">
         <v>67</v>
       </c>
-      <c r="J14" s="22" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -36924,7 +36924,7 @@
       <c r="I15" s="15" t="n">
         <v>59</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-25</t>
         </is>
@@ -36965,7 +36965,7 @@
       <c r="I16" s="20" t="n">
         <v>75</v>
       </c>
-      <c r="J16" s="22" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-34</t>
         </is>
@@ -37006,7 +37006,7 @@
       <c r="I17" s="15" t="n">
         <v>56</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -37047,7 +37047,7 @@
       <c r="I18" s="20" t="n">
         <v>73</v>
       </c>
-      <c r="J18" s="22" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-23</t>
         </is>
@@ -39447,7 +39447,7 @@
       <c r="I10" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J10" s="22" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>-6</t>
         </is>
@@ -39488,7 +39488,7 @@
       <c r="I11" s="15" t="n">
         <v>64</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="24" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -39529,7 +39529,7 @@
       <c r="I12" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J12" s="22" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>-5</t>
         </is>
@@ -39570,7 +39570,7 @@
       <c r="I13" s="15" t="n">
         <v>56</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-10</t>
         </is>
@@ -39611,7 +39611,7 @@
       <c r="I14" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="J14" s="22" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
@@ -39652,7 +39652,7 @@
       <c r="I15" s="15" t="n">
         <v>62</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-23</t>
         </is>
@@ -39693,7 +39693,7 @@
       <c r="I16" s="20" t="n">
         <v>71</v>
       </c>
-      <c r="J16" s="22" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-29</t>
         </is>
@@ -39734,7 +39734,7 @@
       <c r="I17" s="15" t="n">
         <v>71</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-39</t>
         </is>
@@ -39775,7 +39775,7 @@
       <c r="I18" s="20" t="n">
         <v>65</v>
       </c>
-      <c r="J18" s="22" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-32</t>
         </is>
@@ -42175,7 +42175,7 @@
       <c r="I10" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J10" s="22" t="inlineStr">
+      <c r="J10" s="23" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -42216,7 +42216,7 @@
       <c r="I11" s="15" t="n">
         <v>70</v>
       </c>
-      <c r="J11" s="23" t="inlineStr">
+      <c r="J11" s="24" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -42257,7 +42257,7 @@
       <c r="I12" s="20" t="n">
         <v>51</v>
       </c>
-      <c r="J12" s="22" t="inlineStr">
+      <c r="J12" s="23" t="inlineStr">
         <is>
           <t>-11</t>
         </is>
@@ -42298,7 +42298,7 @@
       <c r="I13" s="15" t="n">
         <v>52</v>
       </c>
-      <c r="J13" s="23" t="inlineStr">
+      <c r="J13" s="24" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -42339,7 +42339,7 @@
       <c r="I14" s="20" t="n">
         <v>55</v>
       </c>
-      <c r="J14" s="22" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -42380,7 +42380,7 @@
       <c r="I15" s="15" t="n">
         <v>51</v>
       </c>
-      <c r="J15" s="23" t="inlineStr">
+      <c r="J15" s="24" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -42421,7 +42421,7 @@
       <c r="I16" s="20" t="n">
         <v>48</v>
       </c>
-      <c r="J16" s="22" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -42462,7 +42462,7 @@
       <c r="I17" s="15" t="n">
         <v>67</v>
       </c>
-      <c r="J17" s="23" t="inlineStr">
+      <c r="J17" s="24" t="inlineStr">
         <is>
           <t>-31</t>
         </is>
@@ -42503,7 +42503,7 @@
       <c r="I18" s="20" t="n">
         <v>49</v>
       </c>
-      <c r="J18" s="22" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>-16</t>
         </is>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 01-09-2026 12:26
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  31 August 2026 om 14:55</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  1 September 2026 om 12:26</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  31 August 2026 om 14:55</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  1 September 2026 om 12:26</t>
         </is>
       </c>
     </row>
@@ -16787,9 +16787,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="F16" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="F16" s="36" t="inlineStr">
+        <is>
+          <t>1-4</t>
         </is>
       </c>
       <c r="G16" s="35" t="inlineStr">

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 02-09-2026 12:00
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  1 September 2026 om 12:26</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  2 September 2026 om 12:00</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  1 September 2026 om 12:26</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  2 September 2026 om 12:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 03-09-2026 11:59
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  2 September 2026 om 12:00</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  3 September 2026 om 11:59</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  2 September 2026 om 12:00</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  3 September 2026 om 11:59</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 04-09-2026 12:01
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  3 September 2026 om 11:59</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  4 September 2026 om 12:01</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  3 September 2026 om 11:59</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  4 September 2026 om 12:01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 05-09-2026 11:10
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  4 September 2026 om 12:01</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  5 September 2026 om 11:10</t>
         </is>
       </c>
     </row>
@@ -1396,11 +1396,11 @@
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>SC Heerenveen</t>
+          <t>Sparta Rotterdam</t>
         </is>
       </c>
       <c r="C13" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D13" s="15" t="n">
         <v>1</v>
@@ -1409,25 +1409,25 @@
         <v>2</v>
       </c>
       <c r="F13" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G13" s="16" t="n">
         <v>5</v>
       </c>
       <c r="H13" s="15" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I13" s="15" t="n">
-        <v>6</v>
-      </c>
-      <c r="J13" s="24" t="inlineStr">
-        <is>
-          <t>-1</t>
+        <v>9</v>
+      </c>
+      <c r="J13" s="15" t="inlineStr">
+        <is>
+          <t>0</t>
         </is>
       </c>
       <c r="K13" s="15" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>20%</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="B14" s="19" t="inlineStr">
         <is>
-          <t>Sparta Rotterdam</t>
+          <t>SC Heerenveen</t>
         </is>
       </c>
       <c r="C14" s="20" t="n">
@@ -1447,23 +1447,23 @@
         <v>1</v>
       </c>
       <c r="E14" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="F14" s="20" t="n">
-        <v>2</v>
-      </c>
       <c r="G14" s="21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H14" s="20" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="I14" s="20" t="n">
-        <v>7</v>
-      </c>
-      <c r="J14" s="20" t="inlineStr">
-        <is>
-          <t>0</t>
+        <v>6</v>
+      </c>
+      <c r="J14" s="23" t="inlineStr">
+        <is>
+          <t>-1</t>
         </is>
       </c>
       <c r="K14" s="20" t="inlineStr">
@@ -1482,25 +1482,25 @@
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D15" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E15" s="15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15" s="15" t="n">
         <v>3</v>
       </c>
       <c r="G15" s="16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H15" s="15" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I15" s="15" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J15" s="24" t="inlineStr">
         <is>
@@ -1509,7 +1509,7 @@
       </c>
       <c r="K15" s="15" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>20%</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  4 September 2026 om 12:01</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  5 September 2026 om 11:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Eredivisie bijgewerkt 06-09-2026 11:34
</commit_message>
<xml_diff>
--- a/Eredivisie_Live.xlsx
+++ b/Eredivisie_Live.xlsx
@@ -333,10 +333,10 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -919,7 +919,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  5 September 2026 om 11:10</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Live stand  —  6 September 2026 om 11:34</t>
         </is>
       </c>
     </row>
@@ -986,38 +986,38 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>PSV</t>
         </is>
       </c>
       <c r="C3" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D3" s="5" t="n">
         <v>4</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" s="5" t="n">
         <v>0</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
-          <t>+10</t>
+          <t>+12</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>80%</t>
         </is>
       </c>
     </row>
@@ -1027,29 +1027,29 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>PSV</t>
+          <t>AZ</t>
         </is>
       </c>
       <c r="C4" s="10" t="n">
         <v>4</v>
       </c>
       <c r="D4" s="10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E4" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" s="10" t="n">
         <v>0</v>
       </c>
       <c r="G4" s="11" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H4" s="10" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I4" s="10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J4" s="12" t="inlineStr">
         <is>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>75%</t>
+          <t>100%</t>
         </is>
       </c>
     </row>
@@ -1072,10 +1072,10 @@
         </is>
       </c>
       <c r="C5" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D5" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5" s="10" t="n">
         <v>2</v>
@@ -1084,22 +1084,22 @@
         <v>0</v>
       </c>
       <c r="G5" s="11" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="I5" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J5" s="12" t="inlineStr">
         <is>
-          <t>+4</t>
+          <t>+6</t>
         </is>
       </c>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>60%</t>
         </is>
       </c>
     </row>
@@ -1109,38 +1109,38 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>AFC Ajax</t>
+          <t>SBV Excelsior</t>
         </is>
       </c>
       <c r="C6" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="D6" s="10" t="n">
-        <v>2</v>
-      </c>
       <c r="E6" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="10" t="n">
-        <v>0</v>
-      </c>
       <c r="G6" s="11" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I6" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
-          <t>+6</t>
+          <t>+7</t>
         </is>
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>67%</t>
+          <t>75%</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Go Ahead Eagles</t>
+          <t>AFC Ajax</t>
         </is>
       </c>
       <c r="C7" s="10" t="n">
@@ -1169,14 +1169,14 @@
         <v>7</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I7" s="10" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="J7" s="12" t="inlineStr">
         <is>
-          <t>+2</t>
+          <t>+4</t>
         </is>
       </c>
       <c r="K7" s="10" t="inlineStr">
@@ -1187,11 +1187,11 @@
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Fortuna Sittard</t>
+          <t>FC Twente '65</t>
         </is>
       </c>
       <c r="C8" s="10" t="n">
@@ -1210,14 +1210,14 @@
         <v>7</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I8" s="10" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J8" s="12" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>+4</t>
         </is>
       </c>
       <c r="K8" s="10" t="inlineStr">
@@ -1232,38 +1232,38 @@
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>NEC</t>
+          <t>Go Ahead Eagles</t>
         </is>
       </c>
       <c r="C9" s="15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D9" s="15" t="n">
         <v>2</v>
       </c>
       <c r="E9" s="15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" s="15" t="n">
         <v>1</v>
       </c>
       <c r="G9" s="16" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="I9" s="15" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="J9" s="17" t="inlineStr">
         <is>
-          <t>+4</t>
+          <t>+2</t>
         </is>
       </c>
       <c r="K9" s="15" t="inlineStr">
         <is>
-          <t>67%</t>
+          <t>50%</t>
         </is>
       </c>
     </row>
@@ -1273,79 +1273,79 @@
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>FC Twente '65</t>
+          <t>Fortuna Sittard</t>
         </is>
       </c>
       <c r="C10" s="20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D10" s="20" t="n">
         <v>2</v>
       </c>
       <c r="E10" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" s="20" t="n">
         <v>1</v>
       </c>
       <c r="G10" s="21" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H10" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="I10" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="I10" s="20" t="n">
-        <v>3</v>
-      </c>
       <c r="J10" s="22" t="inlineStr">
         <is>
-          <t>+4</t>
+          <t>+1</t>
         </is>
       </c>
       <c r="K10" s="20" t="inlineStr">
         <is>
-          <t>67%</t>
+          <t>50%</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="13" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>SBV Excelsior</t>
+          <t>FC Groningen</t>
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D11" s="15" t="n">
         <v>2</v>
       </c>
       <c r="E11" s="15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G11" s="16" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H11" s="15" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="I11" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="J11" s="17" t="inlineStr">
-        <is>
-          <t>+4</t>
+        <v>12</v>
+      </c>
+      <c r="J11" s="23" t="inlineStr">
+        <is>
+          <t>-1</t>
         </is>
       </c>
       <c r="K11" s="15" t="inlineStr">
         <is>
-          <t>67%</t>
+          <t>40%</t>
         </is>
       </c>
     </row>
@@ -1355,7 +1355,7 @@
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>FC Groningen</t>
+          <t>NEC</t>
         </is>
       </c>
       <c r="C12" s="20" t="n">
@@ -1377,11 +1377,11 @@
         <v>9</v>
       </c>
       <c r="I12" s="20" t="n">
-        <v>10</v>
-      </c>
-      <c r="J12" s="23" t="inlineStr">
-        <is>
-          <t>-1</t>
+        <v>7</v>
+      </c>
+      <c r="J12" s="22" t="inlineStr">
+        <is>
+          <t>+2</t>
         </is>
       </c>
       <c r="K12" s="20" t="inlineStr">
@@ -1461,7 +1461,7 @@
       <c r="I14" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-1</t>
         </is>
@@ -1502,7 +1502,7 @@
       <c r="I15" s="15" t="n">
         <v>10</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
@@ -1543,7 +1543,7 @@
       <c r="I16" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-5</t>
         </is>
@@ -1560,11 +1560,11 @@
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>Willem II Tilburg</t>
+          <t>ADO Den Haag</t>
         </is>
       </c>
       <c r="C17" s="15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D17" s="15" t="n">
         <v>0</v>
@@ -1573,7 +1573,7 @@
         <v>1</v>
       </c>
       <c r="F17" s="15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G17" s="16" t="n">
         <v>1</v>
@@ -1582,11 +1582,11 @@
         <v>4</v>
       </c>
       <c r="I17" s="15" t="n">
-        <v>10</v>
-      </c>
-      <c r="J17" s="24" t="inlineStr">
-        <is>
-          <t>-6</t>
+        <v>11</v>
+      </c>
+      <c r="J17" s="23" t="inlineStr">
+        <is>
+          <t>-7</t>
         </is>
       </c>
       <c r="K17" s="15" t="inlineStr">
@@ -1601,7 +1601,7 @@
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>ADO Den Haag</t>
+          <t>FC Utrecht</t>
         </is>
       </c>
       <c r="C18" s="20" t="n">
@@ -1620,14 +1620,14 @@
         <v>1</v>
       </c>
       <c r="H18" s="20" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I18" s="20" t="n">
-        <v>11</v>
-      </c>
-      <c r="J18" s="23" t="inlineStr">
-        <is>
-          <t>-7</t>
+        <v>15</v>
+      </c>
+      <c r="J18" s="24" t="inlineStr">
+        <is>
+          <t>-9</t>
         </is>
       </c>
       <c r="K18" s="20" t="inlineStr">
@@ -1642,7 +1642,7 @@
       </c>
       <c r="B19" s="26" t="inlineStr">
         <is>
-          <t>FC Utrecht</t>
+          <t>Willem II Tilburg</t>
         </is>
       </c>
       <c r="C19" s="27" t="n">
@@ -1661,10 +1661,10 @@
         <v>1</v>
       </c>
       <c r="H19" s="27" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I19" s="27" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J19" s="29" t="inlineStr">
         <is>
@@ -4066,7 +4066,7 @@
       <c r="I11" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J11" s="24" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-11</t>
         </is>
@@ -4107,7 +4107,7 @@
       <c r="I12" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -4148,7 +4148,7 @@
       <c r="I13" s="15" t="n">
         <v>58</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-8</t>
         </is>
@@ -4189,7 +4189,7 @@
       <c r="I14" s="20" t="n">
         <v>49</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-6</t>
         </is>
@@ -4230,7 +4230,7 @@
       <c r="I15" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -4271,7 +4271,7 @@
       <c r="I16" s="20" t="n">
         <v>68</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-28</t>
         </is>
@@ -4312,7 +4312,7 @@
       <c r="I17" s="15" t="n">
         <v>55</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -4353,7 +4353,7 @@
       <c r="I18" s="20" t="n">
         <v>68</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-28</t>
         </is>
@@ -6794,7 +6794,7 @@
       <c r="I11" s="15" t="n">
         <v>41</v>
       </c>
-      <c r="J11" s="24" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
@@ -6835,7 +6835,7 @@
       <c r="I12" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
@@ -6917,7 +6917,7 @@
       <c r="I14" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -6958,7 +6958,7 @@
       <c r="I15" s="15" t="n">
         <v>55</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -6999,7 +6999,7 @@
       <c r="I16" s="20" t="n">
         <v>52</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-23</t>
         </is>
@@ -7040,7 +7040,7 @@
       <c r="I17" s="15" t="n">
         <v>51</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-27</t>
         </is>
@@ -7081,7 +7081,7 @@
       <c r="I18" s="20" t="n">
         <v>46</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-12</t>
         </is>
@@ -9440,7 +9440,7 @@
       <c r="I9" s="15" t="n">
         <v>68</v>
       </c>
-      <c r="J9" s="24" t="inlineStr">
+      <c r="J9" s="23" t="inlineStr">
         <is>
           <t>-7</t>
         </is>
@@ -9481,7 +9481,7 @@
       <c r="I10" s="20" t="n">
         <v>41</v>
       </c>
-      <c r="J10" s="23" t="inlineStr">
+      <c r="J10" s="24" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -9522,7 +9522,7 @@
       <c r="I11" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="J11" s="24" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-5</t>
         </is>
@@ -9563,7 +9563,7 @@
       <c r="I12" s="20" t="n">
         <v>72</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -9604,7 +9604,7 @@
       <c r="I13" s="15" t="n">
         <v>73</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -9645,7 +9645,7 @@
       <c r="I14" s="20" t="n">
         <v>63</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-16</t>
         </is>
@@ -9686,7 +9686,7 @@
       <c r="I15" s="15" t="n">
         <v>57</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -9727,7 +9727,7 @@
       <c r="I16" s="20" t="n">
         <v>72</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-31</t>
         </is>
@@ -9768,7 +9768,7 @@
       <c r="I17" s="15" t="n">
         <v>80</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-30</t>
         </is>
@@ -9809,7 +9809,7 @@
       <c r="I18" s="20" t="n">
         <v>79</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-33</t>
         </is>
@@ -12168,7 +12168,7 @@
       <c r="I9" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J9" s="24" t="inlineStr">
+      <c r="J9" s="23" t="inlineStr">
         <is>
           <t>-8</t>
         </is>
@@ -12209,7 +12209,7 @@
       <c r="I10" s="20" t="n">
         <v>53</v>
       </c>
-      <c r="J10" s="23" t="inlineStr">
+      <c r="J10" s="24" t="inlineStr">
         <is>
           <t>-5</t>
         </is>
@@ -12250,7 +12250,7 @@
       <c r="I11" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J11" s="24" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-12</t>
         </is>
@@ -12291,7 +12291,7 @@
       <c r="I12" s="20" t="n">
         <v>64</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -12332,7 +12332,7 @@
       <c r="I13" s="15" t="n">
         <v>56</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -12414,7 +12414,7 @@
       <c r="I15" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -12455,7 +12455,7 @@
       <c r="I16" s="20" t="n">
         <v>57</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-16</t>
         </is>
@@ -12496,7 +12496,7 @@
       <c r="I17" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -12537,7 +12537,7 @@
       <c r="I18" s="20" t="n">
         <v>69</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-27</t>
         </is>
@@ -14896,7 +14896,7 @@
       <c r="I9" s="15" t="n">
         <v>50</v>
       </c>
-      <c r="J9" s="24" t="inlineStr">
+      <c r="J9" s="23" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -15019,7 +15019,7 @@
       <c r="I12" s="20" t="n">
         <v>55</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -15060,7 +15060,7 @@
       <c r="I13" s="15" t="n">
         <v>59</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -15101,7 +15101,7 @@
       <c r="I14" s="20" t="n">
         <v>60</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -15142,7 +15142,7 @@
       <c r="I15" s="15" t="n">
         <v>44</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -15183,7 +15183,7 @@
       <c r="I16" s="20" t="n">
         <v>67</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-28</t>
         </is>
@@ -15224,7 +15224,7 @@
       <c r="I17" s="15" t="n">
         <v>61</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -15265,7 +15265,7 @@
       <c r="I18" s="20" t="n">
         <v>59</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-27</t>
         </is>
@@ -15399,7 +15399,7 @@
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="30" t="inlineStr">
         <is>
-          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  5 September 2026 om 11:10</t>
+          <t>⚽  EREDIVISIE 2025-2026  —  Onderlinge resultaten  —  6 September 2026 om 11:34</t>
         </is>
       </c>
     </row>
@@ -15658,9 +15658,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="M4" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="M4" s="36" t="inlineStr">
+        <is>
+          <t>1-3</t>
         </is>
       </c>
       <c r="N4" s="35" t="inlineStr">
@@ -16409,9 +16409,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="H12" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="H12" s="36" t="inlineStr">
+        <is>
+          <t>1-3</t>
         </is>
       </c>
       <c r="I12" s="35" t="inlineStr">
@@ -17011,9 +17011,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="L18" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="L18" s="38" t="inlineStr">
+        <is>
+          <t>2-2</t>
         </is>
       </c>
       <c r="M18" s="35" t="inlineStr">
@@ -17215,9 +17215,9 @@
           <t>·</t>
         </is>
       </c>
-      <c r="N20" s="35" t="inlineStr">
-        <is>
-          <t>·</t>
+      <c r="N20" s="36" t="inlineStr">
+        <is>
+          <t>0-3</t>
         </is>
       </c>
       <c r="O20" s="35" t="inlineStr">
@@ -19520,7 +19520,7 @@
       <c r="I9" s="15" t="n">
         <v>48</v>
       </c>
-      <c r="J9" s="24" t="inlineStr">
+      <c r="J9" s="23" t="inlineStr">
         <is>
           <t>-7</t>
         </is>
@@ -19643,7 +19643,7 @@
       <c r="I12" s="20" t="n">
         <v>42</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>-5</t>
         </is>
@@ -19684,7 +19684,7 @@
       <c r="I13" s="15" t="n">
         <v>49</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-1</t>
         </is>
@@ -19725,7 +19725,7 @@
       <c r="I14" s="20" t="n">
         <v>61</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -19766,7 +19766,7 @@
       <c r="I15" s="15" t="n">
         <v>64</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -19807,7 +19807,7 @@
       <c r="I16" s="20" t="n">
         <v>55</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-21</t>
         </is>
@@ -19848,7 +19848,7 @@
       <c r="I17" s="15" t="n">
         <v>60</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-26</t>
         </is>
@@ -19889,7 +19889,7 @@
       <c r="I18" s="20" t="n">
         <v>53</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -22289,7 +22289,7 @@
       <c r="I10" s="20" t="n">
         <v>53</v>
       </c>
-      <c r="J10" s="23" t="inlineStr">
+      <c r="J10" s="24" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
@@ -22330,7 +22330,7 @@
       <c r="I11" s="15" t="n">
         <v>50</v>
       </c>
-      <c r="J11" s="24" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
@@ -22412,7 +22412,7 @@
       <c r="I13" s="15" t="n">
         <v>62</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -22453,7 +22453,7 @@
       <c r="I14" s="20" t="n">
         <v>56</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-10</t>
         </is>
@@ -22494,7 +22494,7 @@
       <c r="I15" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -22535,7 +22535,7 @@
       <c r="I16" s="20" t="n">
         <v>64</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -22576,7 +22576,7 @@
       <c r="I17" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-16</t>
         </is>
@@ -22617,7 +22617,7 @@
       <c r="I18" s="20" t="n">
         <v>68</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-32</t>
         </is>
@@ -25058,7 +25058,7 @@
       <c r="I11" s="15" t="n">
         <v>64</v>
       </c>
-      <c r="J11" s="24" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -25099,7 +25099,7 @@
       <c r="I12" s="20" t="n">
         <v>65</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -25140,7 +25140,7 @@
       <c r="I13" s="15" t="n">
         <v>49</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
@@ -25181,7 +25181,7 @@
       <c r="I14" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-10</t>
         </is>
@@ -25222,7 +25222,7 @@
       <c r="I15" s="15" t="n">
         <v>69</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-24</t>
         </is>
@@ -25263,7 +25263,7 @@
       <c r="I16" s="20" t="n">
         <v>59</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -25304,7 +25304,7 @@
       <c r="I17" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-11</t>
         </is>
@@ -25345,7 +25345,7 @@
       <c r="I18" s="20" t="n">
         <v>64</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-20</t>
         </is>
@@ -27704,7 +27704,7 @@
       <c r="I9" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J9" s="24" t="inlineStr">
+      <c r="J9" s="23" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -27745,7 +27745,7 @@
       <c r="I10" s="20" t="n">
         <v>63</v>
       </c>
-      <c r="J10" s="23" t="inlineStr">
+      <c r="J10" s="24" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -27786,7 +27786,7 @@
       <c r="I11" s="15" t="n">
         <v>63</v>
       </c>
-      <c r="J11" s="24" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -27868,7 +27868,7 @@
       <c r="I13" s="15" t="n">
         <v>55</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -27909,7 +27909,7 @@
       <c r="I14" s="20" t="n">
         <v>71</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -27950,7 +27950,7 @@
       <c r="I15" s="15" t="n">
         <v>56</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-16</t>
         </is>
@@ -27991,7 +27991,7 @@
       <c r="I16" s="20" t="n">
         <v>48</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -28032,7 +28032,7 @@
       <c r="I17" s="15" t="n">
         <v>66</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -28073,7 +28073,7 @@
       <c r="I18" s="20" t="n">
         <v>69</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -30473,7 +30473,7 @@
       <c r="I10" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="J10" s="23" t="inlineStr">
+      <c r="J10" s="24" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
@@ -30514,7 +30514,7 @@
       <c r="I11" s="15" t="n">
         <v>49</v>
       </c>
-      <c r="J11" s="24" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -30555,7 +30555,7 @@
       <c r="I12" s="20" t="n">
         <v>70</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -30596,7 +30596,7 @@
       <c r="I13" s="15" t="n">
         <v>58</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
@@ -30637,7 +30637,7 @@
       <c r="I14" s="20" t="n">
         <v>62</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-10</t>
         </is>
@@ -30678,7 +30678,7 @@
       <c r="I15" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-9</t>
         </is>
@@ -30719,7 +30719,7 @@
       <c r="I16" s="20" t="n">
         <v>61</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-20</t>
         </is>
@@ -30760,7 +30760,7 @@
       <c r="I17" s="15" t="n">
         <v>67</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-29</t>
         </is>
@@ -30801,7 +30801,7 @@
       <c r="I18" s="20" t="n">
         <v>78</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-36</t>
         </is>
@@ -31346,7 +31346,7 @@
       <c r="I11" s="15" t="n">
         <v>57</v>
       </c>
-      <c r="J11" s="24" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-15</t>
         </is>
@@ -31387,7 +31387,7 @@
       <c r="I12" s="20" t="n">
         <v>51</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>-8</t>
         </is>
@@ -31428,7 +31428,7 @@
       <c r="I13" s="15" t="n">
         <v>54</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -31469,7 +31469,7 @@
       <c r="I14" s="20" t="n">
         <v>43</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
@@ -31510,7 +31510,7 @@
       <c r="I15" s="15" t="n">
         <v>53</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -31551,7 +31551,7 @@
       <c r="I16" s="20" t="n">
         <v>63</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-21</t>
         </is>
@@ -31592,7 +31592,7 @@
       <c r="I17" s="15" t="n">
         <v>58</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-24</t>
         </is>
@@ -31633,7 +31633,7 @@
       <c r="I18" s="20" t="n">
         <v>56</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -33725,21 +33725,21 @@
       </c>
       <c r="B5" s="45" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>PSV</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>+10</t>
+          <t>+12</t>
         </is>
       </c>
       <c r="H5" s="45" t="inlineStr">
@@ -33785,7 +33785,7 @@
         </is>
       </c>
       <c r="I6" s="18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J6" s="20" t="n">
         <v>14</v>
@@ -33852,17 +33852,6 @@
         <is>
           <t>+51</t>
         </is>
-      </c>
-      <c r="H8" s="48" t="inlineStr">
-        <is>
-          <t>AZ</t>
-        </is>
-      </c>
-      <c r="I8" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" s="20" t="n">
-        <v>14</v>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1">
@@ -36801,7 +36790,7 @@
       <c r="I12" s="20" t="n">
         <v>56</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>-19</t>
         </is>
@@ -36842,7 +36831,7 @@
       <c r="I13" s="15" t="n">
         <v>70</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -36883,7 +36872,7 @@
       <c r="I14" s="20" t="n">
         <v>67</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-22</t>
         </is>
@@ -36924,7 +36913,7 @@
       <c r="I15" s="15" t="n">
         <v>59</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-25</t>
         </is>
@@ -36965,7 +36954,7 @@
       <c r="I16" s="20" t="n">
         <v>75</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-34</t>
         </is>
@@ -37006,7 +36995,7 @@
       <c r="I17" s="15" t="n">
         <v>56</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -37047,7 +37036,7 @@
       <c r="I18" s="20" t="n">
         <v>73</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-23</t>
         </is>
@@ -39447,7 +39436,7 @@
       <c r="I10" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J10" s="23" t="inlineStr">
+      <c r="J10" s="24" t="inlineStr">
         <is>
           <t>-6</t>
         </is>
@@ -39488,7 +39477,7 @@
       <c r="I11" s="15" t="n">
         <v>64</v>
       </c>
-      <c r="J11" s="24" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -39529,7 +39518,7 @@
       <c r="I12" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>-5</t>
         </is>
@@ -39570,7 +39559,7 @@
       <c r="I13" s="15" t="n">
         <v>56</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-10</t>
         </is>
@@ -39611,7 +39600,7 @@
       <c r="I14" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
@@ -39652,7 +39641,7 @@
       <c r="I15" s="15" t="n">
         <v>62</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-23</t>
         </is>
@@ -39693,7 +39682,7 @@
       <c r="I16" s="20" t="n">
         <v>71</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-29</t>
         </is>
@@ -39734,7 +39723,7 @@
       <c r="I17" s="15" t="n">
         <v>71</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-39</t>
         </is>
@@ -39775,7 +39764,7 @@
       <c r="I18" s="20" t="n">
         <v>65</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-32</t>
         </is>
@@ -42175,7 +42164,7 @@
       <c r="I10" s="20" t="n">
         <v>50</v>
       </c>
-      <c r="J10" s="23" t="inlineStr">
+      <c r="J10" s="24" t="inlineStr">
         <is>
           <t>-13</t>
         </is>
@@ -42216,7 +42205,7 @@
       <c r="I11" s="15" t="n">
         <v>70</v>
       </c>
-      <c r="J11" s="24" t="inlineStr">
+      <c r="J11" s="23" t="inlineStr">
         <is>
           <t>-17</t>
         </is>
@@ -42257,7 +42246,7 @@
       <c r="I12" s="20" t="n">
         <v>51</v>
       </c>
-      <c r="J12" s="23" t="inlineStr">
+      <c r="J12" s="24" t="inlineStr">
         <is>
           <t>-11</t>
         </is>
@@ -42298,7 +42287,7 @@
       <c r="I13" s="15" t="n">
         <v>52</v>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -42339,7 +42328,7 @@
       <c r="I14" s="20" t="n">
         <v>55</v>
       </c>
-      <c r="J14" s="23" t="inlineStr">
+      <c r="J14" s="24" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -42380,7 +42369,7 @@
       <c r="I15" s="15" t="n">
         <v>51</v>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-14</t>
         </is>
@@ -42421,7 +42410,7 @@
       <c r="I16" s="20" t="n">
         <v>48</v>
       </c>
-      <c r="J16" s="23" t="inlineStr">
+      <c r="J16" s="24" t="inlineStr">
         <is>
           <t>-18</t>
         </is>
@@ -42462,7 +42451,7 @@
       <c r="I17" s="15" t="n">
         <v>67</v>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="23" t="inlineStr">
         <is>
           <t>-31</t>
         </is>
@@ -42503,7 +42492,7 @@
       <c r="I18" s="20" t="n">
         <v>49</v>
       </c>
-      <c r="J18" s="23" t="inlineStr">
+      <c r="J18" s="24" t="inlineStr">
         <is>
           <t>-16</t>
         </is>

</xml_diff>